<commit_message>
Tasa BCV FIJA, ORDEN DE COMPRA BOLIVARES, FIRMAS AUTORIZADAS POR USUARIO Y ROL
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO ODC CON BOLIVARES.xlsx
+++ b/storage/app/templates/FORMATO ODC CON BOLIVARES.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adv\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA-OFICIAL-AGARCORP\storage\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AAEDDD7-66FC-4F4F-AD7C-5095417BCE78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE35244-E894-4D83-AE8E-77F5323608FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="1" xr2:uid="{CD2C727A-B478-40DC-A0A5-37EBD1630B47}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="54">
   <si>
     <t>TOTAL</t>
   </si>
@@ -191,19 +191,103 @@
     <t>CONTACTO: {{contacto_proveedor}}</t>
   </si>
   <si>
-    <t>EXENTO: {{monto_exento}}</t>
-  </si>
-  <si>
-    <t>SUB-TOTAL: {{sub_total}}</t>
-  </si>
-  <si>
-    <t>IVA 16%: {{iva_16}}</t>
-  </si>
-  <si>
-    <t>GASTOS ADICIONALES: {{gastos_adicionales}}</t>
-  </si>
-  <si>
-    <t>TOTAL: {{total_general}}</t>
+    <t>{{empresa_razon_social}}</t>
+  </si>
+  <si>
+    <t>{{empresa_rif}}</t>
+  </si>
+  <si>
+    <t>{{empresa_telefono_principal}}</t>
+  </si>
+  <si>
+    <t>SITIO DE ENTREGA: {{sitio_entrega}}</t>
+  </si>
+  <si>
+    <t>CONDICIÓN DE PAGO: {{condicion_pago}}</t>
+  </si>
+  <si>
+    <t>COMENTARIOS: {{comentarios}}</t>
+  </si>
+  <si>
+    <t>TASA BCV: {{tasa_bcv}}</t>
+  </si>
+  <si>
+    <t>SOLICITADO POR: {{departamento_solicitante}}</t>
+  </si>
+  <si>
+    <t>ASOCIADO A SUMARIO DE COTIZACIONES N°: {{correlativo_sdc}}</t>
+  </si>
+  <si>
+    <t>ELABORADO POR: {{elaborado_por_nombre}}</t>
+  </si>
+  <si>
+    <t>APROBADO POR: {{aprobado_por_nombre}}</t>
+  </si>
+  <si>
+    <t>CARGO: {{aprobado_por_cargo}}</t>
+  </si>
+  <si>
+    <t>CARGO: {{elaborado_por_cargo}}</t>
+  </si>
+  <si>
+    <t>{{item}}</t>
+  </si>
+  <si>
+    <t>{{descripcion}}</t>
+  </si>
+  <si>
+    <t>{{unidad_medida}}</t>
+  </si>
+  <si>
+    <t>{{cantidad}}</t>
+  </si>
+  <si>
+    <t>{{empresa_direccion_fiscal}}</t>
+  </si>
+  <si>
+    <t>{{precio_unitario}}</t>
+  </si>
+  <si>
+    <t>ORDEN DE COMPRA</t>
+  </si>
+  <si>
+    <t>PROVEEDOR: {{proveedor_nombre}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIRMA: </t>
+  </si>
+  <si>
+    <t>{{firma_elaborado}}</t>
+  </si>
+  <si>
+    <t>{{firma_aprobado}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                  </t>
+  </si>
+  <si>
+    <t>UNITARIO DIVISAS</t>
+  </si>
+  <si>
+    <t>UNITARIO BS</t>
+  </si>
+  <si>
+    <t>{{precio_unitario_bs}}</t>
+  </si>
+  <si>
+    <t>EXENTO: {{monto_exento_bs}}</t>
+  </si>
+  <si>
+    <t>SUB-TOTAL: {{sub_total_bs}}</t>
+  </si>
+  <si>
+    <t>IVA 16%: {{iva_16_bs}}</t>
+  </si>
+  <si>
+    <t>GASTOS ADICIONALES: {{gastos_adicionales_bs}}</t>
+  </si>
+  <si>
+    <t>TOTAL: {{total_general_bs}}</t>
   </si>
   <si>
     <r>
@@ -216,92 +300,11 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>{{total_en_letras}}</t>
+      <t>{{total_en_letras_bs}}</t>
     </r>
   </si>
   <si>
-    <t>{{empresa_razon_social}}</t>
-  </si>
-  <si>
-    <t>{{empresa_rif}}</t>
-  </si>
-  <si>
-    <t>{{empresa_telefono_principal}}</t>
-  </si>
-  <si>
-    <t>SITIO DE ENTREGA: {{sitio_entrega}}</t>
-  </si>
-  <si>
-    <t>CONDICIÓN DE PAGO: {{condicion_pago}}</t>
-  </si>
-  <si>
-    <t>COMENTARIOS: {{comentarios}}</t>
-  </si>
-  <si>
-    <t>TASA BCV: {{tasa_bcv}}</t>
-  </si>
-  <si>
-    <t>SOLICITADO POR: {{departamento_solicitante}}</t>
-  </si>
-  <si>
-    <t>ASOCIADO A SUMARIO DE COTIZACIONES N°: {{correlativo_sdc}}</t>
-  </si>
-  <si>
-    <t>ELABORADO POR: {{elaborado_por_nombre}}</t>
-  </si>
-  <si>
-    <t>APROBADO POR: {{aprobado_por_nombre}}</t>
-  </si>
-  <si>
-    <t>CARGO: {{aprobado_por_cargo}}</t>
-  </si>
-  <si>
-    <t>CARGO: {{elaborado_por_cargo}}</t>
-  </si>
-  <si>
-    <t>{{item}}</t>
-  </si>
-  <si>
-    <t>{{descripcion}}</t>
-  </si>
-  <si>
-    <t>{{unidad_medida}}</t>
-  </si>
-  <si>
-    <t>{{cantidad}}</t>
-  </si>
-  <si>
-    <t>{{empresa_direccion_fiscal}}</t>
-  </si>
-  <si>
-    <t>{{precio_unitario}}</t>
-  </si>
-  <si>
-    <t>{{precio_total}}</t>
-  </si>
-  <si>
-    <t>ORDEN DE COMPRA</t>
-  </si>
-  <si>
-    <t>PROVEEDOR: {{proveedor_nombre}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FIRMA: </t>
-  </si>
-  <si>
-    <t>{{firma_elaborado}}</t>
-  </si>
-  <si>
-    <t>{{firma_aprobado}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">                  </t>
-  </si>
-  <si>
-    <t>UNITARIO DIVISAS</t>
-  </si>
-  <si>
-    <t>UNITARIO BS</t>
+    <t>{{precio_total_bs}}</t>
   </si>
 </sst>
 </file>
@@ -737,12 +740,28 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -773,9 +792,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -920,6 +936,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
@@ -947,22 +966,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="4" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1375,54 +1380,54 @@
   </cols>
   <sheetData>
     <row r="6" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="91"/>
-      <c r="C6" s="94" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="95"/>
-      <c r="E6" s="95"/>
-      <c r="F6" s="96"/>
+      <c r="B6" s="96"/>
+      <c r="C6" s="99" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="100"/>
+      <c r="E6" s="100"/>
+      <c r="F6" s="101"/>
       <c r="G6" s="43"/>
-      <c r="H6" s="54" t="s">
+      <c r="H6" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="55"/>
+      <c r="I6" s="61"/>
     </row>
     <row r="7" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="92"/>
-      <c r="C7" s="97"/>
-      <c r="D7" s="98"/>
-      <c r="E7" s="98"/>
-      <c r="F7" s="99"/>
+      <c r="B7" s="97"/>
+      <c r="C7" s="102"/>
+      <c r="D7" s="103"/>
+      <c r="E7" s="103"/>
+      <c r="F7" s="104"/>
       <c r="G7" s="44"/>
-      <c r="H7" s="54" t="s">
+      <c r="H7" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="I7" s="55"/>
+      <c r="I7" s="61"/>
     </row>
     <row r="8" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="92"/>
-      <c r="C8" s="97"/>
-      <c r="D8" s="98"/>
-      <c r="E8" s="98"/>
-      <c r="F8" s="99"/>
+      <c r="B8" s="97"/>
+      <c r="C8" s="102"/>
+      <c r="D8" s="103"/>
+      <c r="E8" s="103"/>
+      <c r="F8" s="104"/>
       <c r="G8" s="44"/>
-      <c r="H8" s="54" t="s">
+      <c r="H8" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="55"/>
+      <c r="I8" s="61"/>
     </row>
     <row r="9" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="93"/>
-      <c r="C9" s="100"/>
-      <c r="D9" s="101"/>
-      <c r="E9" s="101"/>
-      <c r="F9" s="102"/>
+      <c r="B9" s="98"/>
+      <c r="C9" s="105"/>
+      <c r="D9" s="106"/>
+      <c r="E9" s="106"/>
+      <c r="F9" s="107"/>
       <c r="G9" s="45"/>
-      <c r="H9" s="54" t="s">
+      <c r="H9" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="I9" s="55"/>
+      <c r="I9" s="61"/>
     </row>
     <row r="10" spans="2:9" ht="21" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
@@ -1435,10 +1440,10 @@
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="2:9" ht="43.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="61"/>
+      <c r="B11" s="66" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="67"/>
       <c r="D11" s="16"/>
       <c r="E11" s="17"/>
       <c r="F11" s="17"/>
@@ -1447,38 +1452,38 @@
       <c r="I11" s="19"/>
     </row>
     <row r="12" spans="2:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="62" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="63"/>
+      <c r="B12" s="68" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="69"/>
       <c r="D12" s="20"/>
       <c r="E12" s="21"/>
       <c r="F12" s="22"/>
-      <c r="G12" s="64" t="s">
+      <c r="G12" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="H12" s="64"/>
-      <c r="I12" s="123"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="53"/>
     </row>
     <row r="13" spans="2:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B13" s="32" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C13" s="30"/>
       <c r="D13" s="20"/>
       <c r="E13" s="21"/>
       <c r="F13" s="21"/>
-      <c r="G13" s="64" t="s">
+      <c r="G13" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="H13" s="64"/>
-      <c r="I13" s="123"/>
+      <c r="H13" s="55"/>
+      <c r="I13" s="53"/>
     </row>
     <row r="14" spans="2:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="62" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="63"/>
+      <c r="B14" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="69"/>
       <c r="D14" s="27"/>
       <c r="E14" s="21"/>
       <c r="F14" s="21"/>
@@ -1487,8 +1492,8 @@
       <c r="I14" s="28"/>
     </row>
     <row r="15" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B15" s="65"/>
-      <c r="C15" s="66"/>
+      <c r="B15" s="70"/>
+      <c r="C15" s="71"/>
       <c r="D15" s="29"/>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
@@ -1501,15 +1506,15 @@
     </row>
     <row r="17" spans="2:9" ht="39" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="33" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="56"/>
-      <c r="I17" s="57"/>
+      <c r="F17" s="62"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="62"/>
+      <c r="I17" s="63"/>
     </row>
     <row r="18" spans="2:9" ht="6.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="36"/>
@@ -1529,11 +1534,11 @@
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
       <c r="F19" s="14"/>
-      <c r="G19" s="126" t="s">
+      <c r="G19" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="126"/>
-      <c r="I19" s="127"/>
+      <c r="H19" s="56"/>
+      <c r="I19" s="57"/>
     </row>
     <row r="20" spans="2:9" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="36"/>
@@ -1545,18 +1550,18 @@
       <c r="I20" s="11"/>
     </row>
     <row r="21" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="58" t="s">
+      <c r="B21" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="59"/>
-      <c r="D21" s="59"/>
-      <c r="E21" s="59"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="124" t="s">
+      <c r="C21" s="65"/>
+      <c r="D21" s="65"/>
+      <c r="E21" s="65"/>
+      <c r="F21" s="65"/>
+      <c r="G21" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="H21" s="124"/>
-      <c r="I21" s="128"/>
+      <c r="H21" s="58"/>
+      <c r="I21" s="59"/>
     </row>
     <row r="22" spans="2:9" ht="12.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="12"/>
@@ -1569,16 +1574,16 @@
       <c r="I22" s="13"/>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B23" s="67" t="s">
+      <c r="B23" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="C23" s="68"/>
-      <c r="D23" s="68"/>
-      <c r="E23" s="68"/>
-      <c r="F23" s="68"/>
-      <c r="G23" s="68"/>
-      <c r="H23" s="68"/>
-      <c r="I23" s="69"/>
+      <c r="C23" s="73"/>
+      <c r="D23" s="73"/>
+      <c r="E23" s="73"/>
+      <c r="F23" s="73"/>
+      <c r="G23" s="73"/>
+      <c r="H23" s="73"/>
+      <c r="I23" s="74"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B24" s="12"/>
@@ -1591,15 +1596,15 @@
       <c r="I24" s="13"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B25" s="67" t="s">
+      <c r="B25" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="68"/>
-      <c r="D25" s="68"/>
-      <c r="E25" s="68"/>
-      <c r="F25" s="68"/>
-      <c r="G25" s="68"/>
-      <c r="H25" s="68"/>
+      <c r="C25" s="73"/>
+      <c r="D25" s="73"/>
+      <c r="E25" s="73"/>
+      <c r="F25" s="73"/>
+      <c r="G25" s="73"/>
+      <c r="H25" s="73"/>
       <c r="I25" s="13"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.35">
@@ -1613,16 +1618,16 @@
       <c r="I26" s="13"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B27" s="76" t="s">
+      <c r="B27" s="81" t="s">
         <v>18</v>
       </c>
-      <c r="C27" s="77"/>
-      <c r="D27" s="77"/>
-      <c r="E27" s="77"/>
-      <c r="F27" s="77"/>
-      <c r="G27" s="77"/>
-      <c r="H27" s="77"/>
-      <c r="I27" s="78"/>
+      <c r="C27" s="82"/>
+      <c r="D27" s="82"/>
+      <c r="E27" s="82"/>
+      <c r="F27" s="82"/>
+      <c r="G27" s="82"/>
+      <c r="H27" s="82"/>
+      <c r="I27" s="83"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B28" s="5"/>
@@ -1645,17 +1650,17 @@
       <c r="I29" s="31"/>
     </row>
     <row r="30" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B30" s="71" t="s">
+      <c r="B30" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="C30" s="73" t="s">
+      <c r="C30" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="D30" s="74"/>
-      <c r="E30" s="75" t="s">
+      <c r="D30" s="79"/>
+      <c r="E30" s="80" t="s">
         <v>3</v>
       </c>
-      <c r="F30" s="75" t="s">
+      <c r="F30" s="80" t="s">
         <v>2</v>
       </c>
       <c r="G30" s="4" t="s">
@@ -1669,16 +1674,16 @@
       </c>
     </row>
     <row r="31" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B31" s="72"/>
-      <c r="C31" s="73"/>
-      <c r="D31" s="74"/>
-      <c r="E31" s="75"/>
-      <c r="F31" s="75"/>
+      <c r="B31" s="77"/>
+      <c r="C31" s="78"/>
+      <c r="D31" s="79"/>
+      <c r="E31" s="80"/>
+      <c r="F31" s="80"/>
       <c r="G31" s="4" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H31" s="48" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="I31" s="35" t="s">
         <v>0</v>
@@ -1686,327 +1691,349 @@
     </row>
     <row r="32" spans="2:9" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C32" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D32" s="70"/>
+        <v>32</v>
+      </c>
+      <c r="C32" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="D32" s="75"/>
       <c r="E32" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F32" s="40" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="F32" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="G32" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H32" s="125"/>
+        <v>37</v>
+      </c>
+      <c r="H32" s="128" t="s">
+        <v>46</v>
+      </c>
       <c r="I32" s="41" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="2:9" ht="19.8" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C33" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D33" s="70"/>
+        <v>32</v>
+      </c>
+      <c r="C33" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="D33" s="75"/>
       <c r="E33" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F33" s="40" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="F33" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="G33" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H33" s="125"/>
+        <v>37</v>
+      </c>
+      <c r="H33" s="128" t="s">
+        <v>46</v>
+      </c>
       <c r="I33" s="41" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="2:9" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C34" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D34" s="70"/>
+        <v>32</v>
+      </c>
+      <c r="C34" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="D34" s="75"/>
       <c r="E34" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F34" s="40" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="F34" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="G34" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H34" s="125"/>
+        <v>37</v>
+      </c>
+      <c r="H34" s="128" t="s">
+        <v>46</v>
+      </c>
       <c r="I34" s="41" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="2:9" ht="16.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C35" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D35" s="70"/>
+        <v>32</v>
+      </c>
+      <c r="C35" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="D35" s="75"/>
       <c r="E35" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F35" s="40" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="F35" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="G35" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H35" s="125"/>
+        <v>37</v>
+      </c>
+      <c r="H35" s="128" t="s">
+        <v>46</v>
+      </c>
       <c r="I35" s="41" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B36" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C36" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D36" s="70"/>
+        <v>32</v>
+      </c>
+      <c r="C36" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="D36" s="75"/>
       <c r="E36" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F36" s="40" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="F36" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="G36" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H36" s="125"/>
-      <c r="I36" s="41" t="s">
-        <v>44</v>
+        <v>37</v>
+      </c>
+      <c r="H36" s="128" t="s">
+        <v>46</v>
+      </c>
+      <c r="I36" s="128" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B37" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C37" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D37" s="70"/>
+        <v>32</v>
+      </c>
+      <c r="C37" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="D37" s="75"/>
       <c r="E37" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F37" s="40" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="F37" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="G37" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H37" s="125"/>
-      <c r="I37" s="41" t="s">
-        <v>44</v>
+        <v>37</v>
+      </c>
+      <c r="H37" s="128" t="s">
+        <v>46</v>
+      </c>
+      <c r="I37" s="128" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B38" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C38" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D38" s="70"/>
+        <v>32</v>
+      </c>
+      <c r="C38" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="D38" s="75"/>
       <c r="E38" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F38" s="40" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="F38" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="G38" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H38" s="125"/>
-      <c r="I38" s="41" t="s">
-        <v>44</v>
+        <v>37</v>
+      </c>
+      <c r="H38" s="128" t="s">
+        <v>46</v>
+      </c>
+      <c r="I38" s="128" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B39" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C39" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D39" s="70"/>
+        <v>32</v>
+      </c>
+      <c r="C39" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="D39" s="75"/>
       <c r="E39" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F39" s="40" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="F39" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="G39" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H39" s="125"/>
-      <c r="I39" s="41" t="s">
-        <v>44</v>
+        <v>37</v>
+      </c>
+      <c r="H39" s="128" t="s">
+        <v>46</v>
+      </c>
+      <c r="I39" s="128" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B40" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C40" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D40" s="70"/>
+        <v>32</v>
+      </c>
+      <c r="C40" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="D40" s="75"/>
       <c r="E40" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F40" s="40" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="F40" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="G40" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H40" s="125"/>
-      <c r="I40" s="41" t="s">
-        <v>44</v>
+        <v>37</v>
+      </c>
+      <c r="H40" s="128" t="s">
+        <v>46</v>
+      </c>
+      <c r="I40" s="128" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B41" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C41" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D41" s="70"/>
+        <v>32</v>
+      </c>
+      <c r="C41" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="D41" s="75"/>
       <c r="E41" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F41" s="40" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="F41" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="G41" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H41" s="125"/>
-      <c r="I41" s="41" t="s">
-        <v>44</v>
+        <v>37</v>
+      </c>
+      <c r="H41" s="128" t="s">
+        <v>46</v>
+      </c>
+      <c r="I41" s="128" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B42" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C42" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D42" s="70"/>
+        <v>32</v>
+      </c>
+      <c r="C42" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="D42" s="75"/>
       <c r="E42" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F42" s="40" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="F42" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="G42" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H42" s="125"/>
-      <c r="I42" s="41" t="s">
-        <v>44</v>
+        <v>37</v>
+      </c>
+      <c r="H42" s="128" t="s">
+        <v>46</v>
+      </c>
+      <c r="I42" s="128" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B43" s="109"/>
-      <c r="C43" s="109"/>
-      <c r="D43" s="109"/>
-      <c r="E43" s="109"/>
-      <c r="F43" s="109"/>
-      <c r="G43" s="109"/>
-      <c r="H43" s="109"/>
-      <c r="I43" s="109"/>
+      <c r="B43" s="114"/>
+      <c r="C43" s="114"/>
+      <c r="D43" s="114"/>
+      <c r="E43" s="114"/>
+      <c r="F43" s="114"/>
+      <c r="G43" s="114"/>
+      <c r="H43" s="114"/>
+      <c r="I43" s="114"/>
     </row>
     <row r="44" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B44" s="110"/>
-      <c r="C44" s="111"/>
-      <c r="D44" s="111"/>
-      <c r="E44" s="111"/>
-      <c r="F44" s="112" t="s">
-        <v>19</v>
-      </c>
-      <c r="G44" s="122"/>
-      <c r="H44" s="113"/>
+      <c r="B44" s="115"/>
+      <c r="C44" s="116"/>
+      <c r="D44" s="116"/>
+      <c r="E44" s="116"/>
+      <c r="F44" s="117" t="s">
+        <v>47</v>
+      </c>
+      <c r="G44" s="118"/>
+      <c r="H44" s="119"/>
       <c r="I44" s="8"/>
     </row>
     <row r="45" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B45" s="112" t="s">
-        <v>24</v>
-      </c>
-      <c r="C45" s="113"/>
-      <c r="D45" s="113"/>
-      <c r="E45" s="113"/>
-      <c r="F45" s="112" t="s">
-        <v>20</v>
-      </c>
-      <c r="G45" s="122"/>
-      <c r="H45" s="113"/>
+      <c r="B45" s="117" t="s">
+        <v>52</v>
+      </c>
+      <c r="C45" s="119"/>
+      <c r="D45" s="119"/>
+      <c r="E45" s="119"/>
+      <c r="F45" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="G45" s="118"/>
+      <c r="H45" s="119"/>
       <c r="I45" s="8"/>
     </row>
     <row r="46" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B46" s="103"/>
-      <c r="C46" s="104"/>
-      <c r="D46" s="104"/>
-      <c r="E46" s="105"/>
-      <c r="F46" s="112" t="s">
-        <v>21</v>
-      </c>
-      <c r="G46" s="122"/>
-      <c r="H46" s="113"/>
+      <c r="B46" s="108"/>
+      <c r="C46" s="109"/>
+      <c r="D46" s="109"/>
+      <c r="E46" s="110"/>
+      <c r="F46" s="117" t="s">
+        <v>49</v>
+      </c>
+      <c r="G46" s="118"/>
+      <c r="H46" s="119"/>
       <c r="I46" s="8"/>
     </row>
     <row r="47" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="103"/>
-      <c r="C47" s="104"/>
-      <c r="D47" s="104"/>
-      <c r="E47" s="105"/>
-      <c r="F47" s="118" t="s">
-        <v>22</v>
-      </c>
-      <c r="G47" s="119"/>
-      <c r="H47" s="119"/>
-      <c r="I47" s="120"/>
+      <c r="B47" s="108"/>
+      <c r="C47" s="109"/>
+      <c r="D47" s="109"/>
+      <c r="E47" s="110"/>
+      <c r="F47" s="124" t="s">
+        <v>50</v>
+      </c>
+      <c r="G47" s="125"/>
+      <c r="H47" s="125"/>
+      <c r="I47" s="126"/>
     </row>
     <row r="48" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B48" s="103"/>
-      <c r="C48" s="104"/>
-      <c r="D48" s="104"/>
-      <c r="E48" s="105"/>
-      <c r="F48" s="113" t="s">
-        <v>23</v>
-      </c>
-      <c r="G48" s="113"/>
-      <c r="H48" s="113"/>
+      <c r="B48" s="108"/>
+      <c r="C48" s="109"/>
+      <c r="D48" s="109"/>
+      <c r="E48" s="110"/>
+      <c r="F48" s="119" t="s">
+        <v>51</v>
+      </c>
+      <c r="G48" s="119"/>
+      <c r="H48" s="119"/>
       <c r="I48" s="8"/>
     </row>
     <row r="49" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B49" s="106"/>
-      <c r="C49" s="107"/>
-      <c r="D49" s="107"/>
-      <c r="E49" s="108"/>
-      <c r="F49" s="106"/>
-      <c r="G49" s="107"/>
-      <c r="H49" s="107"/>
-      <c r="I49" s="108"/>
+      <c r="B49" s="111"/>
+      <c r="C49" s="112"/>
+      <c r="D49" s="112"/>
+      <c r="E49" s="113"/>
+      <c r="F49" s="111"/>
+      <c r="G49" s="112"/>
+      <c r="H49" s="112"/>
+      <c r="I49" s="113"/>
     </row>
     <row r="50" spans="2:9" ht="9.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B50" s="42"/>
@@ -2019,20 +2046,20 @@
       <c r="I50" s="19"/>
     </row>
     <row r="51" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B51" s="62" t="s">
-        <v>28</v>
-      </c>
-      <c r="C51" s="63"/>
-      <c r="D51" s="63"/>
-      <c r="E51" s="63"/>
-      <c r="F51" s="63"/>
-      <c r="G51" s="63"/>
-      <c r="H51" s="63"/>
-      <c r="I51" s="121"/>
+      <c r="B51" s="68" t="s">
+        <v>22</v>
+      </c>
+      <c r="C51" s="69"/>
+      <c r="D51" s="69"/>
+      <c r="E51" s="69"/>
+      <c r="F51" s="69"/>
+      <c r="G51" s="69"/>
+      <c r="H51" s="69"/>
+      <c r="I51" s="127"/>
     </row>
     <row r="52" spans="2:9" ht="21" x14ac:dyDescent="0.4">
       <c r="B52" s="37" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C52" s="38"/>
       <c r="D52" s="38"/>
@@ -2043,157 +2070,157 @@
       <c r="I52" s="39"/>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B53" s="117"/>
-      <c r="C53" s="117"/>
-      <c r="D53" s="117"/>
-      <c r="E53" s="117"/>
-      <c r="F53" s="117"/>
-      <c r="G53" s="117"/>
-      <c r="H53" s="117"/>
-      <c r="I53" s="117"/>
+      <c r="B53" s="123"/>
+      <c r="C53" s="123"/>
+      <c r="D53" s="123"/>
+      <c r="E53" s="123"/>
+      <c r="F53" s="123"/>
+      <c r="G53" s="123"/>
+      <c r="H53" s="123"/>
+      <c r="I53" s="123"/>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B54" s="114"/>
-      <c r="C54" s="115"/>
-      <c r="D54" s="115"/>
-      <c r="E54" s="115"/>
-      <c r="F54" s="115"/>
-      <c r="G54" s="115"/>
-      <c r="H54" s="115"/>
-      <c r="I54" s="116"/>
+      <c r="B54" s="120"/>
+      <c r="C54" s="121"/>
+      <c r="D54" s="121"/>
+      <c r="E54" s="121"/>
+      <c r="F54" s="121"/>
+      <c r="G54" s="121"/>
+      <c r="H54" s="121"/>
+      <c r="I54" s="122"/>
     </row>
     <row r="55" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B55" s="62" t="s">
+      <c r="B55" s="68" t="s">
+        <v>24</v>
+      </c>
+      <c r="C55" s="69"/>
+      <c r="D55" s="69"/>
+      <c r="E55" s="69"/>
+      <c r="F55" s="69"/>
+      <c r="G55" s="69"/>
+      <c r="H55" s="69"/>
+      <c r="I55" s="84"/>
+    </row>
+    <row r="56" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B56" s="68"/>
+      <c r="C56" s="69"/>
+      <c r="D56" s="69"/>
+      <c r="E56" s="69"/>
+      <c r="F56" s="69"/>
+      <c r="G56" s="69"/>
+      <c r="H56" s="69"/>
+      <c r="I56" s="84"/>
+    </row>
+    <row r="57" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B57" s="68" t="s">
+        <v>25</v>
+      </c>
+      <c r="C57" s="69"/>
+      <c r="D57" s="69"/>
+      <c r="E57" s="69"/>
+      <c r="F57" s="69"/>
+      <c r="G57" s="69"/>
+      <c r="H57" s="69"/>
+      <c r="I57" s="84"/>
+    </row>
+    <row r="58" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B58" s="68" t="s">
+        <v>26</v>
+      </c>
+      <c r="C58" s="69"/>
+      <c r="D58" s="69"/>
+      <c r="E58" s="69"/>
+      <c r="F58" s="69"/>
+      <c r="G58" s="69"/>
+      <c r="H58" s="69"/>
+      <c r="I58" s="84"/>
+    </row>
+    <row r="59" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B59" s="68" t="s">
+        <v>27</v>
+      </c>
+      <c r="C59" s="69"/>
+      <c r="D59" s="69"/>
+      <c r="E59" s="69"/>
+      <c r="F59" s="69"/>
+      <c r="G59" s="69"/>
+      <c r="H59" s="69"/>
+      <c r="I59" s="84"/>
+    </row>
+    <row r="60" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B60" s="93"/>
+      <c r="C60" s="94"/>
+      <c r="D60" s="94"/>
+      <c r="E60" s="94"/>
+      <c r="F60" s="94"/>
+      <c r="G60" s="94"/>
+      <c r="H60" s="94"/>
+      <c r="I60" s="95"/>
+    </row>
+    <row r="61" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B61" s="86" t="s">
+        <v>28</v>
+      </c>
+      <c r="C61" s="87"/>
+      <c r="D61" s="88"/>
+      <c r="E61" s="88"/>
+      <c r="F61" s="89" t="s">
+        <v>29</v>
+      </c>
+      <c r="G61" s="89"/>
+      <c r="H61" s="89"/>
+      <c r="I61" s="89"/>
+    </row>
+    <row r="62" spans="2:9" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B62" s="86" t="s">
+        <v>31</v>
+      </c>
+      <c r="C62" s="87"/>
+      <c r="D62" s="88"/>
+      <c r="E62" s="88"/>
+      <c r="F62" s="89" t="s">
         <v>30</v>
       </c>
-      <c r="C55" s="63"/>
-      <c r="D55" s="63"/>
-      <c r="E55" s="63"/>
-      <c r="F55" s="63"/>
-      <c r="G55" s="63"/>
-      <c r="H55" s="63"/>
-      <c r="I55" s="79"/>
-    </row>
-    <row r="56" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B56" s="62"/>
-      <c r="C56" s="63"/>
-      <c r="D56" s="63"/>
-      <c r="E56" s="63"/>
-      <c r="F56" s="63"/>
-      <c r="G56" s="63"/>
-      <c r="H56" s="63"/>
-      <c r="I56" s="79"/>
-    </row>
-    <row r="57" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B57" s="62" t="s">
-        <v>31</v>
-      </c>
-      <c r="C57" s="63"/>
-      <c r="D57" s="63"/>
-      <c r="E57" s="63"/>
-      <c r="F57" s="63"/>
-      <c r="G57" s="63"/>
-      <c r="H57" s="63"/>
-      <c r="I57" s="79"/>
-    </row>
-    <row r="58" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B58" s="62" t="s">
-        <v>32</v>
-      </c>
-      <c r="C58" s="63"/>
-      <c r="D58" s="63"/>
-      <c r="E58" s="63"/>
-      <c r="F58" s="63"/>
-      <c r="G58" s="63"/>
-      <c r="H58" s="63"/>
-      <c r="I58" s="79"/>
-    </row>
-    <row r="59" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B59" s="62" t="s">
-        <v>33</v>
-      </c>
-      <c r="C59" s="63"/>
-      <c r="D59" s="63"/>
-      <c r="E59" s="63"/>
-      <c r="F59" s="63"/>
-      <c r="G59" s="63"/>
-      <c r="H59" s="63"/>
-      <c r="I59" s="79"/>
-    </row>
-    <row r="60" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B60" s="88"/>
-      <c r="C60" s="89"/>
-      <c r="D60" s="89"/>
-      <c r="E60" s="89"/>
-      <c r="F60" s="89"/>
-      <c r="G60" s="89"/>
-      <c r="H60" s="89"/>
-      <c r="I60" s="90"/>
-    </row>
-    <row r="61" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B61" s="81" t="s">
-        <v>34</v>
-      </c>
-      <c r="C61" s="82"/>
-      <c r="D61" s="83"/>
-      <c r="E61" s="83"/>
-      <c r="F61" s="84" t="s">
-        <v>35</v>
-      </c>
-      <c r="G61" s="84"/>
-      <c r="H61" s="84"/>
-      <c r="I61" s="84"/>
-    </row>
-    <row r="62" spans="2:9" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B62" s="81" t="s">
-        <v>37</v>
-      </c>
-      <c r="C62" s="82"/>
-      <c r="D62" s="83"/>
-      <c r="E62" s="83"/>
-      <c r="F62" s="84" t="s">
-        <v>36</v>
-      </c>
-      <c r="G62" s="84"/>
-      <c r="H62" s="84"/>
-      <c r="I62" s="84"/>
+      <c r="G62" s="89"/>
+      <c r="H62" s="89"/>
+      <c r="I62" s="89"/>
     </row>
     <row r="63" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="42" t="s">
-        <v>48</v>
-      </c>
-      <c r="C63" s="52"/>
-      <c r="D63" s="83"/>
-      <c r="E63" s="83"/>
+      <c r="B63" s="42"/>
+      <c r="C63" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D63" s="88"/>
+      <c r="E63" s="88"/>
       <c r="F63" s="51" t="s">
-        <v>50</v>
-      </c>
-      <c r="G63" s="53" t="s">
-        <v>49</v>
+        <v>43</v>
+      </c>
+      <c r="G63" s="52" t="s">
+        <v>42</v>
       </c>
       <c r="I63" s="50"/>
     </row>
     <row r="64" spans="2:9" ht="51.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B64" s="85" t="s">
-        <v>47</v>
-      </c>
-      <c r="C64" s="86"/>
-      <c r="D64" s="83"/>
-      <c r="E64" s="83"/>
-      <c r="F64" s="87" t="s">
-        <v>47</v>
-      </c>
-      <c r="G64" s="87"/>
-      <c r="H64" s="87"/>
-      <c r="I64" s="87"/>
+      <c r="B64" s="90" t="s">
+        <v>40</v>
+      </c>
+      <c r="C64" s="91"/>
+      <c r="D64" s="88"/>
+      <c r="E64" s="88"/>
+      <c r="F64" s="92" t="s">
+        <v>40</v>
+      </c>
+      <c r="G64" s="92"/>
+      <c r="H64" s="92"/>
+      <c r="I64" s="92"/>
     </row>
     <row r="65" spans="4:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="D65" s="80"/>
-      <c r="E65" s="80"/>
+      <c r="D65" s="85"/>
+      <c r="E65" s="85"/>
     </row>
     <row r="66" spans="4:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="D66" s="80"/>
-      <c r="E66" s="80"/>
+      <c r="D66" s="85"/>
+      <c r="E66" s="85"/>
     </row>
   </sheetData>
   <mergeCells count="65">
@@ -2204,20 +2231,16 @@
     <mergeCell ref="C33:D33"/>
     <mergeCell ref="B51:I51"/>
     <mergeCell ref="C42:D42"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="C6:F9"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="F44:H44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="F45:H45"/>
     <mergeCell ref="B46:E46"/>
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="B49:E49"/>
     <mergeCell ref="B48:E48"/>
     <mergeCell ref="F49:I49"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="B43:I43"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="F44:H44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="F45:H45"/>
     <mergeCell ref="F46:H46"/>
     <mergeCell ref="F48:H48"/>
     <mergeCell ref="B56:I56"/>
@@ -2248,11 +2271,8 @@
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C38:D38"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="G19:I19"/>
@@ -2262,6 +2282,13 @@
     <mergeCell ref="H8:I8"/>
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="F17:I17"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="C6:F9"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="49" orientation="portrait" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Logo y firmas enviadas mas abajo en odc, se ve mal en win10 pero bien en ubuntu
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO ODC CON BOLIVARES.xlsx
+++ b/storage/app/templates/FORMATO ODC CON BOLIVARES.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA-OFICIAL-AGARCORP\storage\app\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adv\AppData\Roaming\MobaXterm\slash\mx86_64b\RemoteFiles\3146582_3_8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE35244-E894-4D83-AE8E-77F5323608FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35D1B80B-DB99-46CB-B53C-2B9D06E555E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="1" xr2:uid="{CD2C727A-B478-40DC-A0A5-37EBD1630B47}"/>
   </bookViews>
@@ -747,6 +747,147 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="4" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -786,90 +927,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -904,69 +967,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -995,14 +995,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>241300</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>257592</xdr:rowOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>202177</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>1612900</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>228599</xdr:rowOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>173184</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1032,8 +1032,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="2019300" y="1527592"/>
-          <a:ext cx="1371600" cy="1114007"/>
+          <a:off x="2028536" y="1906286"/>
+          <a:ext cx="1371600" cy="1134789"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1364,7 +1364,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B6:I66"/>
+  <dimension ref="B6:I68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="26" defaultRowHeight="20.399999999999999" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26" style="1"/>
@@ -1380,54 +1380,54 @@
   </cols>
   <sheetData>
     <row r="6" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="96"/>
-      <c r="C6" s="99" t="s">
+      <c r="B6" s="117"/>
+      <c r="C6" s="120" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="100"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="101"/>
+      <c r="D6" s="121"/>
+      <c r="E6" s="121"/>
+      <c r="F6" s="122"/>
       <c r="G6" s="43"/>
-      <c r="H6" s="60" t="s">
+      <c r="H6" s="107" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="61"/>
+      <c r="I6" s="108"/>
     </row>
     <row r="7" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="97"/>
-      <c r="C7" s="102"/>
-      <c r="D7" s="103"/>
-      <c r="E7" s="103"/>
-      <c r="F7" s="104"/>
+      <c r="B7" s="118"/>
+      <c r="C7" s="123"/>
+      <c r="D7" s="124"/>
+      <c r="E7" s="124"/>
+      <c r="F7" s="125"/>
       <c r="G7" s="44"/>
-      <c r="H7" s="60" t="s">
+      <c r="H7" s="107" t="s">
         <v>8</v>
       </c>
-      <c r="I7" s="61"/>
+      <c r="I7" s="108"/>
     </row>
     <row r="8" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="97"/>
-      <c r="C8" s="102"/>
-      <c r="D8" s="103"/>
-      <c r="E8" s="103"/>
-      <c r="F8" s="104"/>
+      <c r="B8" s="118"/>
+      <c r="C8" s="123"/>
+      <c r="D8" s="124"/>
+      <c r="E8" s="124"/>
+      <c r="F8" s="125"/>
       <c r="G8" s="44"/>
-      <c r="H8" s="60" t="s">
+      <c r="H8" s="107" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="61"/>
+      <c r="I8" s="108"/>
     </row>
     <row r="9" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="98"/>
-      <c r="C9" s="105"/>
-      <c r="D9" s="106"/>
-      <c r="E9" s="106"/>
-      <c r="F9" s="107"/>
+      <c r="B9" s="119"/>
+      <c r="C9" s="126"/>
+      <c r="D9" s="127"/>
+      <c r="E9" s="127"/>
+      <c r="F9" s="128"/>
       <c r="G9" s="45"/>
-      <c r="H9" s="60" t="s">
+      <c r="H9" s="107" t="s">
         <v>6</v>
       </c>
-      <c r="I9" s="61"/>
+      <c r="I9" s="108"/>
     </row>
     <row r="10" spans="2:9" ht="21" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
@@ -1440,10 +1440,10 @@
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="2:9" ht="43.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="66" t="s">
+      <c r="B11" s="113" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="67"/>
+      <c r="C11" s="114"/>
       <c r="D11" s="16"/>
       <c r="E11" s="17"/>
       <c r="F11" s="17"/>
@@ -1452,17 +1452,17 @@
       <c r="I11" s="19"/>
     </row>
     <row r="12" spans="2:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="68" t="s">
+      <c r="B12" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="69"/>
+      <c r="C12" s="57"/>
       <c r="D12" s="20"/>
       <c r="E12" s="21"/>
       <c r="F12" s="22"/>
-      <c r="G12" s="55" t="s">
+      <c r="G12" s="102" t="s">
         <v>10</v>
       </c>
-      <c r="H12" s="55"/>
+      <c r="H12" s="102"/>
       <c r="I12" s="53"/>
     </row>
     <row r="13" spans="2:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.4">
@@ -1473,17 +1473,17 @@
       <c r="D13" s="20"/>
       <c r="E13" s="21"/>
       <c r="F13" s="21"/>
-      <c r="G13" s="55" t="s">
+      <c r="G13" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="H13" s="55"/>
+      <c r="H13" s="102"/>
       <c r="I13" s="53"/>
     </row>
     <row r="14" spans="2:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="68" t="s">
+      <c r="B14" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="69"/>
+      <c r="C14" s="57"/>
       <c r="D14" s="27"/>
       <c r="E14" s="21"/>
       <c r="F14" s="21"/>
@@ -1492,8 +1492,8 @@
       <c r="I14" s="28"/>
     </row>
     <row r="15" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B15" s="70"/>
-      <c r="C15" s="71"/>
+      <c r="B15" s="115"/>
+      <c r="C15" s="116"/>
       <c r="D15" s="29"/>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
@@ -1511,10 +1511,10 @@
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
-      <c r="F17" s="62"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="62"/>
-      <c r="I17" s="63"/>
+      <c r="F17" s="109"/>
+      <c r="G17" s="109"/>
+      <c r="H17" s="109"/>
+      <c r="I17" s="110"/>
     </row>
     <row r="18" spans="2:9" ht="6.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="36"/>
@@ -1534,11 +1534,11 @@
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
       <c r="F19" s="14"/>
-      <c r="G19" s="56" t="s">
+      <c r="G19" s="103" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="56"/>
-      <c r="I19" s="57"/>
+      <c r="H19" s="103"/>
+      <c r="I19" s="104"/>
     </row>
     <row r="20" spans="2:9" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="36"/>
@@ -1550,18 +1550,18 @@
       <c r="I20" s="11"/>
     </row>
     <row r="21" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="64" t="s">
+      <c r="B21" s="111" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="65"/>
-      <c r="D21" s="65"/>
-      <c r="E21" s="65"/>
-      <c r="F21" s="65"/>
-      <c r="G21" s="58" t="s">
+      <c r="C21" s="112"/>
+      <c r="D21" s="112"/>
+      <c r="E21" s="112"/>
+      <c r="F21" s="112"/>
+      <c r="G21" s="105" t="s">
         <v>15</v>
       </c>
-      <c r="H21" s="58"/>
-      <c r="I21" s="59"/>
+      <c r="H21" s="105"/>
+      <c r="I21" s="106"/>
     </row>
     <row r="22" spans="2:9" ht="12.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="12"/>
@@ -1574,16 +1574,16 @@
       <c r="I22" s="13"/>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B23" s="72" t="s">
+      <c r="B23" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="C23" s="73"/>
-      <c r="D23" s="73"/>
-      <c r="E23" s="73"/>
-      <c r="F23" s="73"/>
-      <c r="G23" s="73"/>
-      <c r="H23" s="73"/>
-      <c r="I23" s="74"/>
+      <c r="C23" s="92"/>
+      <c r="D23" s="92"/>
+      <c r="E23" s="92"/>
+      <c r="F23" s="92"/>
+      <c r="G23" s="92"/>
+      <c r="H23" s="92"/>
+      <c r="I23" s="93"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B24" s="12"/>
@@ -1596,15 +1596,15 @@
       <c r="I24" s="13"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B25" s="72" t="s">
+      <c r="B25" s="91" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="73"/>
-      <c r="D25" s="73"/>
-      <c r="E25" s="73"/>
-      <c r="F25" s="73"/>
-      <c r="G25" s="73"/>
-      <c r="H25" s="73"/>
+      <c r="C25" s="92"/>
+      <c r="D25" s="92"/>
+      <c r="E25" s="92"/>
+      <c r="F25" s="92"/>
+      <c r="G25" s="92"/>
+      <c r="H25" s="92"/>
       <c r="I25" s="13"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.35">
@@ -1618,16 +1618,16 @@
       <c r="I26" s="13"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B27" s="81" t="s">
+      <c r="B27" s="99" t="s">
         <v>18</v>
       </c>
-      <c r="C27" s="82"/>
-      <c r="D27" s="82"/>
-      <c r="E27" s="82"/>
-      <c r="F27" s="82"/>
-      <c r="G27" s="82"/>
-      <c r="H27" s="82"/>
-      <c r="I27" s="83"/>
+      <c r="C27" s="100"/>
+      <c r="D27" s="100"/>
+      <c r="E27" s="100"/>
+      <c r="F27" s="100"/>
+      <c r="G27" s="100"/>
+      <c r="H27" s="100"/>
+      <c r="I27" s="101"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B28" s="5"/>
@@ -1650,17 +1650,17 @@
       <c r="I29" s="31"/>
     </row>
     <row r="30" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B30" s="76" t="s">
+      <c r="B30" s="94" t="s">
         <v>5</v>
       </c>
-      <c r="C30" s="78" t="s">
+      <c r="C30" s="96" t="s">
         <v>4</v>
       </c>
-      <c r="D30" s="79"/>
-      <c r="E30" s="80" t="s">
+      <c r="D30" s="97"/>
+      <c r="E30" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="F30" s="80" t="s">
+      <c r="F30" s="98" t="s">
         <v>2</v>
       </c>
       <c r="G30" s="4" t="s">
@@ -1674,11 +1674,11 @@
       </c>
     </row>
     <row r="31" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B31" s="77"/>
-      <c r="C31" s="78"/>
-      <c r="D31" s="79"/>
-      <c r="E31" s="80"/>
-      <c r="F31" s="80"/>
+      <c r="B31" s="95"/>
+      <c r="C31" s="96"/>
+      <c r="D31" s="97"/>
+      <c r="E31" s="98"/>
+      <c r="F31" s="98"/>
       <c r="G31" s="4" t="s">
         <v>44</v>
       </c>
@@ -1693,10 +1693,10 @@
       <c r="B32" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C32" s="75" t="s">
+      <c r="C32" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D32" s="75"/>
+      <c r="D32" s="66"/>
       <c r="E32" s="40" t="s">
         <v>35</v>
       </c>
@@ -1706,7 +1706,7 @@
       <c r="G32" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H32" s="128" t="s">
+      <c r="H32" s="55" t="s">
         <v>46</v>
       </c>
       <c r="I32" s="41" t="s">
@@ -1717,10 +1717,10 @@
       <c r="B33" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="75" t="s">
+      <c r="C33" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D33" s="75"/>
+      <c r="D33" s="66"/>
       <c r="E33" s="40" t="s">
         <v>35</v>
       </c>
@@ -1730,7 +1730,7 @@
       <c r="G33" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H33" s="128" t="s">
+      <c r="H33" s="55" t="s">
         <v>46</v>
       </c>
       <c r="I33" s="41" t="s">
@@ -1741,10 +1741,10 @@
       <c r="B34" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C34" s="75" t="s">
+      <c r="C34" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D34" s="75"/>
+      <c r="D34" s="66"/>
       <c r="E34" s="40" t="s">
         <v>35</v>
       </c>
@@ -1754,7 +1754,7 @@
       <c r="G34" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H34" s="128" t="s">
+      <c r="H34" s="55" t="s">
         <v>46</v>
       </c>
       <c r="I34" s="41" t="s">
@@ -1765,10 +1765,10 @@
       <c r="B35" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C35" s="75" t="s">
+      <c r="C35" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D35" s="75"/>
+      <c r="D35" s="66"/>
       <c r="E35" s="40" t="s">
         <v>35</v>
       </c>
@@ -1778,7 +1778,7 @@
       <c r="G35" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H35" s="128" t="s">
+      <c r="H35" s="55" t="s">
         <v>46</v>
       </c>
       <c r="I35" s="41" t="s">
@@ -1789,10 +1789,10 @@
       <c r="B36" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C36" s="75" t="s">
+      <c r="C36" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D36" s="75"/>
+      <c r="D36" s="66"/>
       <c r="E36" s="40" t="s">
         <v>35</v>
       </c>
@@ -1802,10 +1802,10 @@
       <c r="G36" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H36" s="128" t="s">
+      <c r="H36" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="I36" s="128" t="s">
+      <c r="I36" s="55" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1813,10 +1813,10 @@
       <c r="B37" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C37" s="75" t="s">
+      <c r="C37" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D37" s="75"/>
+      <c r="D37" s="66"/>
       <c r="E37" s="40" t="s">
         <v>35</v>
       </c>
@@ -1826,10 +1826,10 @@
       <c r="G37" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H37" s="128" t="s">
+      <c r="H37" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="I37" s="128" t="s">
+      <c r="I37" s="55" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1837,10 +1837,10 @@
       <c r="B38" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C38" s="75" t="s">
+      <c r="C38" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D38" s="75"/>
+      <c r="D38" s="66"/>
       <c r="E38" s="40" t="s">
         <v>35</v>
       </c>
@@ -1850,10 +1850,10 @@
       <c r="G38" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H38" s="128" t="s">
+      <c r="H38" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="I38" s="128" t="s">
+      <c r="I38" s="55" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1861,10 +1861,10 @@
       <c r="B39" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C39" s="75" t="s">
+      <c r="C39" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D39" s="75"/>
+      <c r="D39" s="66"/>
       <c r="E39" s="40" t="s">
         <v>35</v>
       </c>
@@ -1874,10 +1874,10 @@
       <c r="G39" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H39" s="128" t="s">
+      <c r="H39" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="I39" s="128" t="s">
+      <c r="I39" s="55" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1885,10 +1885,10 @@
       <c r="B40" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C40" s="75" t="s">
+      <c r="C40" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D40" s="75"/>
+      <c r="D40" s="66"/>
       <c r="E40" s="40" t="s">
         <v>35</v>
       </c>
@@ -1898,10 +1898,10 @@
       <c r="G40" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H40" s="128" t="s">
+      <c r="H40" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="I40" s="128" t="s">
+      <c r="I40" s="55" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1909,10 +1909,10 @@
       <c r="B41" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="75" t="s">
+      <c r="C41" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D41" s="75"/>
+      <c r="D41" s="66"/>
       <c r="E41" s="40" t="s">
         <v>35</v>
       </c>
@@ -1922,10 +1922,10 @@
       <c r="G41" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H41" s="128" t="s">
+      <c r="H41" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="I41" s="128" t="s">
+      <c r="I41" s="55" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1933,10 +1933,10 @@
       <c r="B42" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C42" s="75" t="s">
+      <c r="C42" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D42" s="75"/>
+      <c r="D42" s="66"/>
       <c r="E42" s="40" t="s">
         <v>35</v>
       </c>
@@ -1946,94 +1946,94 @@
       <c r="G42" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H42" s="128" t="s">
+      <c r="H42" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="I42" s="128" t="s">
+      <c r="I42" s="55" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B43" s="114"/>
-      <c r="C43" s="114"/>
-      <c r="D43" s="114"/>
-      <c r="E43" s="114"/>
-      <c r="F43" s="114"/>
-      <c r="G43" s="114"/>
-      <c r="H43" s="114"/>
-      <c r="I43" s="114"/>
+      <c r="B43" s="68"/>
+      <c r="C43" s="68"/>
+      <c r="D43" s="68"/>
+      <c r="E43" s="68"/>
+      <c r="F43" s="68"/>
+      <c r="G43" s="68"/>
+      <c r="H43" s="68"/>
+      <c r="I43" s="68"/>
     </row>
     <row r="44" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B44" s="115"/>
-      <c r="C44" s="116"/>
-      <c r="D44" s="116"/>
-      <c r="E44" s="116"/>
-      <c r="F44" s="117" t="s">
+      <c r="B44" s="69"/>
+      <c r="C44" s="70"/>
+      <c r="D44" s="70"/>
+      <c r="E44" s="70"/>
+      <c r="F44" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="G44" s="118"/>
-      <c r="H44" s="119"/>
+      <c r="G44" s="72"/>
+      <c r="H44" s="73"/>
       <c r="I44" s="8"/>
     </row>
     <row r="45" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B45" s="117" t="s">
+      <c r="B45" s="71" t="s">
         <v>52</v>
       </c>
-      <c r="C45" s="119"/>
-      <c r="D45" s="119"/>
-      <c r="E45" s="119"/>
-      <c r="F45" s="117" t="s">
+      <c r="C45" s="73"/>
+      <c r="D45" s="73"/>
+      <c r="E45" s="73"/>
+      <c r="F45" s="71" t="s">
         <v>48</v>
       </c>
-      <c r="G45" s="118"/>
-      <c r="H45" s="119"/>
+      <c r="G45" s="72"/>
+      <c r="H45" s="73"/>
       <c r="I45" s="8"/>
     </row>
     <row r="46" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B46" s="108"/>
-      <c r="C46" s="109"/>
-      <c r="D46" s="109"/>
-      <c r="E46" s="110"/>
-      <c r="F46" s="117" t="s">
+      <c r="B46" s="74"/>
+      <c r="C46" s="75"/>
+      <c r="D46" s="75"/>
+      <c r="E46" s="76"/>
+      <c r="F46" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="G46" s="118"/>
-      <c r="H46" s="119"/>
+      <c r="G46" s="72"/>
+      <c r="H46" s="73"/>
       <c r="I46" s="8"/>
     </row>
     <row r="47" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="108"/>
-      <c r="C47" s="109"/>
-      <c r="D47" s="109"/>
-      <c r="E47" s="110"/>
-      <c r="F47" s="124" t="s">
+      <c r="B47" s="74"/>
+      <c r="C47" s="75"/>
+      <c r="D47" s="75"/>
+      <c r="E47" s="76"/>
+      <c r="F47" s="63" t="s">
         <v>50</v>
       </c>
-      <c r="G47" s="125"/>
-      <c r="H47" s="125"/>
-      <c r="I47" s="126"/>
+      <c r="G47" s="64"/>
+      <c r="H47" s="64"/>
+      <c r="I47" s="65"/>
     </row>
     <row r="48" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B48" s="108"/>
-      <c r="C48" s="109"/>
-      <c r="D48" s="109"/>
-      <c r="E48" s="110"/>
-      <c r="F48" s="119" t="s">
+      <c r="B48" s="74"/>
+      <c r="C48" s="75"/>
+      <c r="D48" s="75"/>
+      <c r="E48" s="76"/>
+      <c r="F48" s="73" t="s">
         <v>51</v>
       </c>
-      <c r="G48" s="119"/>
-      <c r="H48" s="119"/>
+      <c r="G48" s="73"/>
+      <c r="H48" s="73"/>
       <c r="I48" s="8"/>
     </row>
     <row r="49" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B49" s="111"/>
-      <c r="C49" s="112"/>
-      <c r="D49" s="112"/>
-      <c r="E49" s="113"/>
-      <c r="F49" s="111"/>
-      <c r="G49" s="112"/>
-      <c r="H49" s="112"/>
-      <c r="I49" s="113"/>
+      <c r="B49" s="77"/>
+      <c r="C49" s="78"/>
+      <c r="D49" s="78"/>
+      <c r="E49" s="79"/>
+      <c r="F49" s="77"/>
+      <c r="G49" s="78"/>
+      <c r="H49" s="78"/>
+      <c r="I49" s="79"/>
     </row>
     <row r="50" spans="2:9" ht="9.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B50" s="42"/>
@@ -2046,16 +2046,16 @@
       <c r="I50" s="19"/>
     </row>
     <row r="51" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B51" s="68" t="s">
+      <c r="B51" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="C51" s="69"/>
-      <c r="D51" s="69"/>
-      <c r="E51" s="69"/>
-      <c r="F51" s="69"/>
-      <c r="G51" s="69"/>
-      <c r="H51" s="69"/>
-      <c r="I51" s="127"/>
+      <c r="C51" s="57"/>
+      <c r="D51" s="57"/>
+      <c r="E51" s="57"/>
+      <c r="F51" s="57"/>
+      <c r="G51" s="57"/>
+      <c r="H51" s="57"/>
+      <c r="I51" s="67"/>
     </row>
     <row r="52" spans="2:9" ht="21" x14ac:dyDescent="0.4">
       <c r="B52" s="37" t="s">
@@ -2070,160 +2070,211 @@
       <c r="I52" s="39"/>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B53" s="123"/>
-      <c r="C53" s="123"/>
-      <c r="D53" s="123"/>
-      <c r="E53" s="123"/>
-      <c r="F53" s="123"/>
-      <c r="G53" s="123"/>
-      <c r="H53" s="123"/>
-      <c r="I53" s="123"/>
+      <c r="B53" s="62"/>
+      <c r="C53" s="62"/>
+      <c r="D53" s="62"/>
+      <c r="E53" s="62"/>
+      <c r="F53" s="62"/>
+      <c r="G53" s="62"/>
+      <c r="H53" s="62"/>
+      <c r="I53" s="62"/>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B54" s="120"/>
-      <c r="C54" s="121"/>
-      <c r="D54" s="121"/>
-      <c r="E54" s="121"/>
-      <c r="F54" s="121"/>
-      <c r="G54" s="121"/>
-      <c r="H54" s="121"/>
-      <c r="I54" s="122"/>
+      <c r="B54" s="59"/>
+      <c r="C54" s="60"/>
+      <c r="D54" s="60"/>
+      <c r="E54" s="60"/>
+      <c r="F54" s="60"/>
+      <c r="G54" s="60"/>
+      <c r="H54" s="60"/>
+      <c r="I54" s="61"/>
     </row>
     <row r="55" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B55" s="68" t="s">
+      <c r="B55" s="56" t="s">
         <v>24</v>
       </c>
-      <c r="C55" s="69"/>
-      <c r="D55" s="69"/>
-      <c r="E55" s="69"/>
-      <c r="F55" s="69"/>
-      <c r="G55" s="69"/>
-      <c r="H55" s="69"/>
-      <c r="I55" s="84"/>
+      <c r="C55" s="57"/>
+      <c r="D55" s="57"/>
+      <c r="E55" s="57"/>
+      <c r="F55" s="57"/>
+      <c r="G55" s="57"/>
+      <c r="H55" s="57"/>
+      <c r="I55" s="58"/>
     </row>
     <row r="56" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B56" s="68"/>
-      <c r="C56" s="69"/>
-      <c r="D56" s="69"/>
-      <c r="E56" s="69"/>
-      <c r="F56" s="69"/>
-      <c r="G56" s="69"/>
-      <c r="H56" s="69"/>
-      <c r="I56" s="84"/>
+      <c r="B56" s="56"/>
+      <c r="C56" s="57"/>
+      <c r="D56" s="57"/>
+      <c r="E56" s="57"/>
+      <c r="F56" s="57"/>
+      <c r="G56" s="57"/>
+      <c r="H56" s="57"/>
+      <c r="I56" s="58"/>
     </row>
     <row r="57" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B57" s="68" t="s">
+      <c r="B57" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="C57" s="69"/>
-      <c r="D57" s="69"/>
-      <c r="E57" s="69"/>
-      <c r="F57" s="69"/>
-      <c r="G57" s="69"/>
-      <c r="H57" s="69"/>
-      <c r="I57" s="84"/>
+      <c r="C57" s="57"/>
+      <c r="D57" s="57"/>
+      <c r="E57" s="57"/>
+      <c r="F57" s="57"/>
+      <c r="G57" s="57"/>
+      <c r="H57" s="57"/>
+      <c r="I57" s="58"/>
     </row>
     <row r="58" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B58" s="68" t="s">
+      <c r="B58" s="56" t="s">
         <v>26</v>
       </c>
-      <c r="C58" s="69"/>
-      <c r="D58" s="69"/>
-      <c r="E58" s="69"/>
-      <c r="F58" s="69"/>
-      <c r="G58" s="69"/>
-      <c r="H58" s="69"/>
-      <c r="I58" s="84"/>
+      <c r="C58" s="57"/>
+      <c r="D58" s="57"/>
+      <c r="E58" s="57"/>
+      <c r="F58" s="57"/>
+      <c r="G58" s="57"/>
+      <c r="H58" s="57"/>
+      <c r="I58" s="58"/>
     </row>
     <row r="59" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B59" s="68" t="s">
+      <c r="B59" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="C59" s="69"/>
-      <c r="D59" s="69"/>
-      <c r="E59" s="69"/>
-      <c r="F59" s="69"/>
-      <c r="G59" s="69"/>
-      <c r="H59" s="69"/>
-      <c r="I59" s="84"/>
+      <c r="C59" s="57"/>
+      <c r="D59" s="57"/>
+      <c r="E59" s="57"/>
+      <c r="F59" s="57"/>
+      <c r="G59" s="57"/>
+      <c r="H59" s="57"/>
+      <c r="I59" s="58"/>
     </row>
     <row r="60" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B60" s="93"/>
-      <c r="C60" s="94"/>
-      <c r="D60" s="94"/>
-      <c r="E60" s="94"/>
-      <c r="F60" s="94"/>
-      <c r="G60" s="94"/>
-      <c r="H60" s="94"/>
-      <c r="I60" s="95"/>
+      <c r="B60" s="88"/>
+      <c r="C60" s="89"/>
+      <c r="D60" s="89"/>
+      <c r="E60" s="89"/>
+      <c r="F60" s="89"/>
+      <c r="G60" s="89"/>
+      <c r="H60" s="89"/>
+      <c r="I60" s="90"/>
     </row>
     <row r="61" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B61" s="86" t="s">
+      <c r="B61" s="81" t="s">
         <v>28</v>
       </c>
-      <c r="C61" s="87"/>
-      <c r="D61" s="88"/>
-      <c r="E61" s="88"/>
-      <c r="F61" s="89" t="s">
+      <c r="C61" s="82"/>
+      <c r="D61" s="83"/>
+      <c r="E61" s="83"/>
+      <c r="F61" s="84" t="s">
         <v>29</v>
       </c>
-      <c r="G61" s="89"/>
-      <c r="H61" s="89"/>
-      <c r="I61" s="89"/>
+      <c r="G61" s="84"/>
+      <c r="H61" s="84"/>
+      <c r="I61" s="84"/>
     </row>
     <row r="62" spans="2:9" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B62" s="86" t="s">
+      <c r="B62" s="81" t="s">
         <v>31</v>
       </c>
-      <c r="C62" s="87"/>
-      <c r="D62" s="88"/>
-      <c r="E62" s="88"/>
-      <c r="F62" s="89" t="s">
+      <c r="C62" s="82"/>
+      <c r="D62" s="83"/>
+      <c r="E62" s="83"/>
+      <c r="F62" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="G62" s="89"/>
-      <c r="H62" s="89"/>
-      <c r="I62" s="89"/>
+      <c r="G62" s="84"/>
+      <c r="H62" s="84"/>
+      <c r="I62" s="84"/>
     </row>
     <row r="63" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B63" s="42"/>
-      <c r="C63" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D63" s="88"/>
-      <c r="E63" s="88"/>
+      <c r="D63" s="83"/>
+      <c r="E63" s="83"/>
       <c r="F63" s="51" t="s">
         <v>43</v>
       </c>
-      <c r="G63" s="52" t="s">
+      <c r="I63" s="50"/>
+    </row>
+    <row r="64" spans="2:9" ht="51.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B64" s="85" t="s">
+        <v>40</v>
+      </c>
+      <c r="C64" s="86"/>
+      <c r="D64" s="83"/>
+      <c r="E64" s="83"/>
+      <c r="F64" s="87" t="s">
+        <v>40</v>
+      </c>
+      <c r="G64" s="87"/>
+      <c r="H64" s="87"/>
+      <c r="I64" s="87"/>
+    </row>
+    <row r="65" spans="3:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="D65" s="80"/>
+      <c r="E65" s="80"/>
+    </row>
+    <row r="66" spans="3:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="D66" s="80"/>
+      <c r="E66" s="80"/>
+    </row>
+    <row r="68" spans="3:7" x14ac:dyDescent="0.35">
+      <c r="C68" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="G68" s="52" t="s">
         <v>42</v>
       </c>
-      <c r="I63" s="50"/>
-    </row>
-    <row r="64" spans="2:9" ht="51.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B64" s="90" t="s">
-        <v>40</v>
-      </c>
-      <c r="C64" s="91"/>
-      <c r="D64" s="88"/>
-      <c r="E64" s="88"/>
-      <c r="F64" s="92" t="s">
-        <v>40</v>
-      </c>
-      <c r="G64" s="92"/>
-      <c r="H64" s="92"/>
-      <c r="I64" s="92"/>
-    </row>
-    <row r="65" spans="4:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="D65" s="85"/>
-      <c r="E65" s="85"/>
-    </row>
-    <row r="66" spans="4:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="D66" s="85"/>
-      <c r="E66" s="85"/>
     </row>
   </sheetData>
   <mergeCells count="65">
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="C6:F9"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B59:I59"/>
+    <mergeCell ref="B60:I60"/>
+    <mergeCell ref="B57:I57"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:D31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="D61:E64"/>
+    <mergeCell ref="F61:I61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="F62:I62"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="F64:I64"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="F46:H46"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="B56:I56"/>
+    <mergeCell ref="B58:I58"/>
     <mergeCell ref="B55:I55"/>
     <mergeCell ref="B54:I54"/>
     <mergeCell ref="B53:I53"/>
@@ -2240,55 +2291,6 @@
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="B49:E49"/>
     <mergeCell ref="B48:E48"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="F46:H46"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="B56:I56"/>
-    <mergeCell ref="B58:I58"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="D61:E64"/>
-    <mergeCell ref="F61:I61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="F62:I62"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="F64:I64"/>
-    <mergeCell ref="B59:I59"/>
-    <mergeCell ref="B60:I60"/>
-    <mergeCell ref="B57:I57"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:D31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="F30:F31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="C6:F9"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="49" orientation="portrait" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Correcciones de exportaciones, subida de archivos en Docker y firma agregada
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO ODC CON BOLIVARES.xlsx
+++ b/storage/app/templates/FORMATO ODC CON BOLIVARES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adv\AppData\Roaming\MobaXterm\slash\mx86_64b\RemoteFiles\3146582_3_8\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\AppData\Roaming\MobaXterm\slash\RemoteFiles\66904_6_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35D1B80B-DB99-46CB-B53C-2B9D06E555E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09236216-7662-46AB-B395-10165D64E97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="1" xr2:uid="{CD2C727A-B478-40DC-A0A5-37EBD1630B47}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{CD2C727A-B478-40DC-A0A5-37EBD1630B47}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -41,13 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="54">
-  <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
-    <t>VALOR</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="53">
   <si>
     <t>UNIDAD MED</t>
   </si>
@@ -266,12 +260,6 @@
     <t xml:space="preserve">                  </t>
   </si>
   <si>
-    <t>UNITARIO DIVISAS</t>
-  </si>
-  <si>
-    <t>UNITARIO BS</t>
-  </si>
-  <si>
     <t>{{precio_unitario_bs}}</t>
   </si>
   <si>
@@ -305,6 +293,15 @@
   </si>
   <si>
     <t>{{precio_total_bs}}</t>
+  </si>
+  <si>
+    <t>VALOR UNITARIO DIVISAS</t>
+  </si>
+  <si>
+    <t>VALOR UNITARIO BS</t>
+  </si>
+  <si>
+    <t>VALOR TOTAL</t>
   </si>
 </sst>
 </file>
@@ -385,6 +382,7 @@
     </font>
     <font>
       <b/>
+      <u/>
       <sz val="24"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -615,7 +613,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -623,9 +621,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -690,12 +685,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -713,23 +702,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -750,6 +727,36 @@
     <xf numFmtId="4" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -780,29 +787,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -813,15 +799,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -903,24 +880,24 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -945,28 +922,28 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -994,15 +971,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>241300</xdr:colOff>
+      <xdr:colOff>144316</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>202177</xdr:rowOff>
+      <xdr:rowOff>202178</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1612900</xdr:colOff>
+      <xdr:colOff>1474048</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>173184</xdr:rowOff>
+      <xdr:rowOff>138546</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1032,8 +1009,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="2028536" y="1906286"/>
-          <a:ext cx="1371600" cy="1134789"/>
+          <a:off x="1931552" y="1906287"/>
+          <a:ext cx="1329732" cy="1100150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1380,54 +1357,54 @@
   </cols>
   <sheetData>
     <row r="6" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="117"/>
-      <c r="C6" s="120" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" s="121"/>
-      <c r="E6" s="121"/>
-      <c r="F6" s="122"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="107" t="s">
-        <v>9</v>
-      </c>
-      <c r="I6" s="108"/>
+      <c r="B6" s="110"/>
+      <c r="C6" s="113" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="114"/>
+      <c r="E6" s="114"/>
+      <c r="F6" s="114"/>
+      <c r="G6" s="115"/>
+      <c r="H6" s="102" t="s">
+        <v>7</v>
+      </c>
+      <c r="I6" s="103"/>
     </row>
     <row r="7" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="118"/>
-      <c r="C7" s="123"/>
-      <c r="D7" s="124"/>
-      <c r="E7" s="124"/>
-      <c r="F7" s="125"/>
-      <c r="G7" s="44"/>
-      <c r="H7" s="107" t="s">
-        <v>8</v>
-      </c>
-      <c r="I7" s="108"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="117"/>
+      <c r="E7" s="117"/>
+      <c r="F7" s="117"/>
+      <c r="G7" s="118"/>
+      <c r="H7" s="102" t="s">
+        <v>6</v>
+      </c>
+      <c r="I7" s="103"/>
     </row>
     <row r="8" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="118"/>
-      <c r="C8" s="123"/>
-      <c r="D8" s="124"/>
-      <c r="E8" s="124"/>
-      <c r="F8" s="125"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="107" t="s">
-        <v>7</v>
-      </c>
-      <c r="I8" s="108"/>
+      <c r="B8" s="111"/>
+      <c r="C8" s="116"/>
+      <c r="D8" s="117"/>
+      <c r="E8" s="117"/>
+      <c r="F8" s="117"/>
+      <c r="G8" s="118"/>
+      <c r="H8" s="102" t="s">
+        <v>5</v>
+      </c>
+      <c r="I8" s="103"/>
     </row>
     <row r="9" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="119"/>
-      <c r="C9" s="126"/>
-      <c r="D9" s="127"/>
-      <c r="E9" s="127"/>
-      <c r="F9" s="128"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="107" t="s">
-        <v>6</v>
-      </c>
-      <c r="I9" s="108"/>
+      <c r="B9" s="112"/>
+      <c r="C9" s="119"/>
+      <c r="D9" s="120"/>
+      <c r="E9" s="120"/>
+      <c r="F9" s="120"/>
+      <c r="G9" s="121"/>
+      <c r="H9" s="102" t="s">
+        <v>4</v>
+      </c>
+      <c r="I9" s="103"/>
     </row>
     <row r="10" spans="2:9" ht="21" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
@@ -1435,803 +1412,797 @@
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
-      <c r="G10" s="46"/>
+      <c r="G10" s="40"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="2:9" ht="43.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="113" t="s">
+      <c r="B11" s="106" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="107"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="18"/>
+    </row>
+    <row r="12" spans="2:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="60"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="95" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" s="95"/>
+      <c r="I12" s="46"/>
+    </row>
+    <row r="13" spans="2:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B13" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="29"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="95" t="s">
+        <v>9</v>
+      </c>
+      <c r="H13" s="95"/>
+      <c r="I13" s="46"/>
+    </row>
+    <row r="14" spans="2:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="114"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="19"/>
-    </row>
-    <row r="12" spans="2:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="56" t="s">
+      <c r="C14" s="60"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="27"/>
+    </row>
+    <row r="15" spans="2:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="B15" s="108"/>
+      <c r="C15" s="109"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="24"/>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B16" s="30"/>
+    </row>
+    <row r="17" spans="2:9" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="104"/>
+      <c r="G17" s="104"/>
+      <c r="H17" s="104"/>
+      <c r="I17" s="105"/>
+    </row>
+    <row r="18" spans="2:9" ht="6.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="33"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="10"/>
+    </row>
+    <row r="19" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="96" t="s">
+        <v>11</v>
+      </c>
+      <c r="H19" s="96"/>
+      <c r="I19" s="97"/>
+    </row>
+    <row r="20" spans="2:9" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="33"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="I20" s="10"/>
+    </row>
+    <row r="21" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="100" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="101"/>
+      <c r="D21" s="101"/>
+      <c r="E21" s="101"/>
+      <c r="F21" s="101"/>
+      <c r="G21" s="98" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="98"/>
+      <c r="I21" s="99"/>
+    </row>
+    <row r="22" spans="2:9" ht="12.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="11"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="12"/>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B23" s="84" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="85"/>
+      <c r="D23" s="85"/>
+      <c r="E23" s="85"/>
+      <c r="F23" s="85"/>
+      <c r="G23" s="85"/>
+      <c r="H23" s="85"/>
+      <c r="I23" s="86"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B24" s="11"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="12"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B25" s="84" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="85"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="85"/>
+      <c r="F25" s="85"/>
+      <c r="G25" s="85"/>
+      <c r="H25" s="85"/>
+      <c r="I25" s="12"/>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B26" s="11"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="41"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="12"/>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B27" s="92" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="93"/>
+      <c r="D27" s="93"/>
+      <c r="E27" s="93"/>
+      <c r="F27" s="93"/>
+      <c r="G27" s="93"/>
+      <c r="H27" s="93"/>
+      <c r="I27" s="94"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B28" s="4"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="6"/>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
+    </row>
+    <row r="30" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="87" t="s">
+        <v>3</v>
+      </c>
+      <c r="C30" s="89" t="s">
+        <v>2</v>
+      </c>
+      <c r="D30" s="90"/>
+      <c r="E30" s="91" t="s">
+        <v>1</v>
+      </c>
+      <c r="F30" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="G30" s="87" t="s">
+        <v>50</v>
+      </c>
+      <c r="H30" s="87" t="s">
+        <v>51</v>
+      </c>
+      <c r="I30" s="87" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" ht="45.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B31" s="88"/>
+      <c r="C31" s="89"/>
+      <c r="D31" s="90"/>
+      <c r="E31" s="91"/>
+      <c r="F31" s="91"/>
+      <c r="G31" s="88"/>
+      <c r="H31" s="88"/>
+      <c r="I31" s="88"/>
+    </row>
+    <row r="32" spans="2:9" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B32" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D32" s="49"/>
+      <c r="E32" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F32" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G32" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H32" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="I32" s="38" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" ht="19.8" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D33" s="49"/>
+      <c r="E33" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F33" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G33" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H33" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="I33" s="38" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B34" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C34" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D34" s="49"/>
+      <c r="E34" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F34" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G34" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H34" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="I34" s="38" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" ht="16.2" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B35" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D35" s="49"/>
+      <c r="E35" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F35" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G35" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H35" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="I35" s="38" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B36" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D36" s="49"/>
+      <c r="E36" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F36" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G36" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H36" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="I36" s="48" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B37" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D37" s="49"/>
+      <c r="E37" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F37" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G37" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H37" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="I37" s="48" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B38" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C38" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D38" s="49"/>
+      <c r="E38" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F38" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G38" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H38" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="I38" s="48" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B39" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C39" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D39" s="49"/>
+      <c r="E39" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F39" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G39" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H39" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="I39" s="48" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B40" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C40" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D40" s="49"/>
+      <c r="E40" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F40" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G40" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H40" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="I40" s="48" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B41" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D41" s="49"/>
+      <c r="E41" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F41" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G41" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H41" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="I41" s="48" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B42" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C42" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D42" s="49"/>
+      <c r="E42" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F42" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G42" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H42" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="I42" s="48" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B43" s="50"/>
+      <c r="C43" s="50"/>
+      <c r="D43" s="50"/>
+      <c r="E43" s="50"/>
+      <c r="F43" s="50"/>
+      <c r="G43" s="50"/>
+      <c r="H43" s="50"/>
+      <c r="I43" s="50"/>
+    </row>
+    <row r="44" spans="2:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="B44" s="51"/>
+      <c r="C44" s="52"/>
+      <c r="D44" s="52"/>
+      <c r="E44" s="52"/>
+      <c r="F44" s="53" t="s">
+        <v>43</v>
+      </c>
+      <c r="G44" s="54"/>
+      <c r="H44" s="55"/>
+      <c r="I44" s="7"/>
+    </row>
+    <row r="45" spans="2:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="B45" s="53" t="s">
+        <v>48</v>
+      </c>
+      <c r="C45" s="55"/>
+      <c r="D45" s="55"/>
+      <c r="E45" s="55"/>
+      <c r="F45" s="53" t="s">
+        <v>44</v>
+      </c>
+      <c r="G45" s="54"/>
+      <c r="H45" s="55"/>
+      <c r="I45" s="7"/>
+    </row>
+    <row r="46" spans="2:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="B46" s="70"/>
+      <c r="C46" s="71"/>
+      <c r="D46" s="71"/>
+      <c r="E46" s="72"/>
+      <c r="F46" s="53" t="s">
+        <v>45</v>
+      </c>
+      <c r="G46" s="54"/>
+      <c r="H46" s="55"/>
+      <c r="I46" s="7"/>
+    </row>
+    <row r="47" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B47" s="70"/>
+      <c r="C47" s="71"/>
+      <c r="D47" s="71"/>
+      <c r="E47" s="72"/>
+      <c r="F47" s="66" t="s">
+        <v>46</v>
+      </c>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="68"/>
+    </row>
+    <row r="48" spans="2:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="B48" s="70"/>
+      <c r="C48" s="71"/>
+      <c r="D48" s="71"/>
+      <c r="E48" s="72"/>
+      <c r="F48" s="55" t="s">
+        <v>47</v>
+      </c>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="7"/>
+    </row>
+    <row r="49" spans="2:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="B49" s="56"/>
+      <c r="C49" s="57"/>
+      <c r="D49" s="57"/>
+      <c r="E49" s="58"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="57"/>
+      <c r="H49" s="57"/>
+      <c r="I49" s="58"/>
+    </row>
+    <row r="50" spans="2:9" ht="9.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B50" s="39"/>
+      <c r="C50" s="17"/>
+      <c r="D50" s="17"/>
+      <c r="E50" s="17"/>
+      <c r="F50" s="17"/>
+      <c r="G50" s="17"/>
+      <c r="H50" s="17"/>
+      <c r="I50" s="18"/>
+    </row>
+    <row r="51" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B51" s="59" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="57"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="102" t="s">
-        <v>10</v>
-      </c>
-      <c r="H12" s="102"/>
-      <c r="I12" s="53"/>
-    </row>
-    <row r="13" spans="2:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="102" t="s">
-        <v>11</v>
-      </c>
-      <c r="H13" s="102"/>
-      <c r="I13" s="53"/>
-    </row>
-    <row r="14" spans="2:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="56" t="s">
+      <c r="C51" s="60"/>
+      <c r="D51" s="60"/>
+      <c r="E51" s="60"/>
+      <c r="F51" s="60"/>
+      <c r="G51" s="60"/>
+      <c r="H51" s="60"/>
+      <c r="I51" s="69"/>
+    </row>
+    <row r="52" spans="2:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="B52" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="57"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="28"/>
-    </row>
-    <row r="15" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B15" s="115"/>
-      <c r="C15" s="116"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="25"/>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B16" s="31"/>
-    </row>
-    <row r="17" spans="2:9" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="33" t="s">
+      <c r="C52" s="35"/>
+      <c r="D52" s="35"/>
+      <c r="E52" s="35"/>
+      <c r="F52" s="35"/>
+      <c r="G52" s="35"/>
+      <c r="H52" s="35"/>
+      <c r="I52" s="36"/>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B53" s="65"/>
+      <c r="C53" s="65"/>
+      <c r="D53" s="65"/>
+      <c r="E53" s="65"/>
+      <c r="F53" s="65"/>
+      <c r="G53" s="65"/>
+      <c r="H53" s="65"/>
+      <c r="I53" s="65"/>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B54" s="62"/>
+      <c r="C54" s="63"/>
+      <c r="D54" s="63"/>
+      <c r="E54" s="63"/>
+      <c r="F54" s="63"/>
+      <c r="G54" s="63"/>
+      <c r="H54" s="63"/>
+      <c r="I54" s="64"/>
+    </row>
+    <row r="55" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B55" s="59" t="s">
+        <v>22</v>
+      </c>
+      <c r="C55" s="60"/>
+      <c r="D55" s="60"/>
+      <c r="E55" s="60"/>
+      <c r="F55" s="60"/>
+      <c r="G55" s="60"/>
+      <c r="H55" s="60"/>
+      <c r="I55" s="61"/>
+    </row>
+    <row r="56" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B56" s="59"/>
+      <c r="C56" s="60"/>
+      <c r="D56" s="60"/>
+      <c r="E56" s="60"/>
+      <c r="F56" s="60"/>
+      <c r="G56" s="60"/>
+      <c r="H56" s="60"/>
+      <c r="I56" s="61"/>
+    </row>
+    <row r="57" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B57" s="59" t="s">
+        <v>23</v>
+      </c>
+      <c r="C57" s="60"/>
+      <c r="D57" s="60"/>
+      <c r="E57" s="60"/>
+      <c r="F57" s="60"/>
+      <c r="G57" s="60"/>
+      <c r="H57" s="60"/>
+      <c r="I57" s="61"/>
+    </row>
+    <row r="58" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B58" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="C58" s="60"/>
+      <c r="D58" s="60"/>
+      <c r="E58" s="60"/>
+      <c r="F58" s="60"/>
+      <c r="G58" s="60"/>
+      <c r="H58" s="60"/>
+      <c r="I58" s="61"/>
+    </row>
+    <row r="59" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B59" s="59" t="s">
+        <v>25</v>
+      </c>
+      <c r="C59" s="60"/>
+      <c r="D59" s="60"/>
+      <c r="E59" s="60"/>
+      <c r="F59" s="60"/>
+      <c r="G59" s="60"/>
+      <c r="H59" s="60"/>
+      <c r="I59" s="61"/>
+    </row>
+    <row r="60" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="B60" s="81"/>
+      <c r="C60" s="82"/>
+      <c r="D60" s="82"/>
+      <c r="E60" s="82"/>
+      <c r="F60" s="82"/>
+      <c r="G60" s="82"/>
+      <c r="H60" s="82"/>
+      <c r="I60" s="83"/>
+    </row>
+    <row r="61" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B61" s="74" t="s">
+        <v>26</v>
+      </c>
+      <c r="C61" s="75"/>
+      <c r="D61" s="76"/>
+      <c r="E61" s="76"/>
+      <c r="F61" s="77" t="s">
+        <v>27</v>
+      </c>
+      <c r="G61" s="77"/>
+      <c r="H61" s="77"/>
+      <c r="I61" s="77"/>
+    </row>
+    <row r="62" spans="2:9" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B62" s="74" t="s">
+        <v>29</v>
+      </c>
+      <c r="C62" s="75"/>
+      <c r="D62" s="76"/>
+      <c r="E62" s="76"/>
+      <c r="F62" s="77" t="s">
+        <v>28</v>
+      </c>
+      <c r="G62" s="77"/>
+      <c r="H62" s="77"/>
+      <c r="I62" s="77"/>
+    </row>
+    <row r="63" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B63" s="39"/>
+      <c r="D63" s="76"/>
+      <c r="E63" s="76"/>
+      <c r="F63" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="I63" s="43"/>
+    </row>
+    <row r="64" spans="2:9" ht="51.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B64" s="78" t="s">
+        <v>38</v>
+      </c>
+      <c r="C64" s="79"/>
+      <c r="D64" s="76"/>
+      <c r="E64" s="76"/>
+      <c r="F64" s="80" t="s">
+        <v>38</v>
+      </c>
+      <c r="G64" s="80"/>
+      <c r="H64" s="80"/>
+      <c r="I64" s="80"/>
+    </row>
+    <row r="65" spans="3:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="D65" s="73"/>
+      <c r="E65" s="73"/>
+    </row>
+    <row r="66" spans="3:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="D66" s="73"/>
+      <c r="E66" s="73"/>
+    </row>
+    <row r="68" spans="3:7" x14ac:dyDescent="0.35">
+      <c r="C68" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="109"/>
-      <c r="G17" s="109"/>
-      <c r="H17" s="109"/>
-      <c r="I17" s="110"/>
-    </row>
-    <row r="18" spans="2:9" ht="6.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="36"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="49"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="11"/>
-    </row>
-    <row r="19" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="103" t="s">
-        <v>13</v>
-      </c>
-      <c r="H19" s="103"/>
-      <c r="I19" s="104"/>
-    </row>
-    <row r="20" spans="2:9" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="36"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="I20" s="11"/>
-    </row>
-    <row r="21" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="111" t="s">
-        <v>14</v>
-      </c>
-      <c r="C21" s="112"/>
-      <c r="D21" s="112"/>
-      <c r="E21" s="112"/>
-      <c r="F21" s="112"/>
-      <c r="G21" s="105" t="s">
-        <v>15</v>
-      </c>
-      <c r="H21" s="105"/>
-      <c r="I21" s="106"/>
-    </row>
-    <row r="22" spans="2:9" ht="12.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="12"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="47"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="13"/>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B23" s="91" t="s">
-        <v>16</v>
-      </c>
-      <c r="C23" s="92"/>
-      <c r="D23" s="92"/>
-      <c r="E23" s="92"/>
-      <c r="F23" s="92"/>
-      <c r="G23" s="92"/>
-      <c r="H23" s="92"/>
-      <c r="I23" s="93"/>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B24" s="12"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="47"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="13"/>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B25" s="91" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="92"/>
-      <c r="D25" s="92"/>
-      <c r="E25" s="92"/>
-      <c r="F25" s="92"/>
-      <c r="G25" s="92"/>
-      <c r="H25" s="92"/>
-      <c r="I25" s="13"/>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B26" s="12"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="47"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="13"/>
-    </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B27" s="99" t="s">
-        <v>18</v>
-      </c>
-      <c r="C27" s="100"/>
-      <c r="D27" s="100"/>
-      <c r="E27" s="100"/>
-      <c r="F27" s="100"/>
-      <c r="G27" s="100"/>
-      <c r="H27" s="100"/>
-      <c r="I27" s="101"/>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B28" s="5"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="7"/>
-    </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="31"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="31"/>
-      <c r="I29" s="31"/>
-    </row>
-    <row r="30" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B30" s="94" t="s">
-        <v>5</v>
-      </c>
-      <c r="C30" s="96" t="s">
-        <v>4</v>
-      </c>
-      <c r="D30" s="97"/>
-      <c r="E30" s="98" t="s">
-        <v>3</v>
-      </c>
-      <c r="F30" s="98" t="s">
-        <v>2</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H30" s="48" t="s">
-        <v>1</v>
-      </c>
-      <c r="I30" s="34" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B31" s="95"/>
-      <c r="C31" s="96"/>
-      <c r="D31" s="97"/>
-      <c r="E31" s="98"/>
-      <c r="F31" s="98"/>
-      <c r="G31" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="H31" s="48" t="s">
-        <v>45</v>
-      </c>
-      <c r="I31" s="35" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="2:9" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="C32" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="D32" s="66"/>
-      <c r="E32" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="F32" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="G32" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H32" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="I32" s="41" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="33" spans="2:9" ht="19.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="C33" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="D33" s="66"/>
-      <c r="E33" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="F33" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="G33" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H33" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="I33" s="41" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="34" spans="2:9" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="C34" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="D34" s="66"/>
-      <c r="E34" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="F34" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="G34" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H34" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="I34" s="41" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="35" spans="2:9" ht="16.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="D35" s="66"/>
-      <c r="E35" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="F35" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="G35" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H35" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="I35" s="41" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B36" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="C36" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="D36" s="66"/>
-      <c r="E36" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="F36" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="G36" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H36" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="I36" s="55" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B37" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="C37" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="D37" s="66"/>
-      <c r="E37" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="F37" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="G37" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H37" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="I37" s="55" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B38" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="C38" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="D38" s="66"/>
-      <c r="E38" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="F38" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="G38" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H38" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="I38" s="55" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B39" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="C39" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="D39" s="66"/>
-      <c r="E39" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="F39" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="G39" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H39" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="I39" s="55" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B40" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="C40" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="D40" s="66"/>
-      <c r="E40" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="F40" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="G40" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H40" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="I40" s="55" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B41" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="C41" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="D41" s="66"/>
-      <c r="E41" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="F41" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="G41" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H41" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="I41" s="55" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B42" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="C42" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="D42" s="66"/>
-      <c r="E42" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="F42" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="G42" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H42" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="I42" s="55" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B43" s="68"/>
-      <c r="C43" s="68"/>
-      <c r="D43" s="68"/>
-      <c r="E43" s="68"/>
-      <c r="F43" s="68"/>
-      <c r="G43" s="68"/>
-      <c r="H43" s="68"/>
-      <c r="I43" s="68"/>
-    </row>
-    <row r="44" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B44" s="69"/>
-      <c r="C44" s="70"/>
-      <c r="D44" s="70"/>
-      <c r="E44" s="70"/>
-      <c r="F44" s="71" t="s">
-        <v>47</v>
-      </c>
-      <c r="G44" s="72"/>
-      <c r="H44" s="73"/>
-      <c r="I44" s="8"/>
-    </row>
-    <row r="45" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B45" s="71" t="s">
-        <v>52</v>
-      </c>
-      <c r="C45" s="73"/>
-      <c r="D45" s="73"/>
-      <c r="E45" s="73"/>
-      <c r="F45" s="71" t="s">
-        <v>48</v>
-      </c>
-      <c r="G45" s="72"/>
-      <c r="H45" s="73"/>
-      <c r="I45" s="8"/>
-    </row>
-    <row r="46" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B46" s="74"/>
-      <c r="C46" s="75"/>
-      <c r="D46" s="75"/>
-      <c r="E46" s="76"/>
-      <c r="F46" s="71" t="s">
-        <v>49</v>
-      </c>
-      <c r="G46" s="72"/>
-      <c r="H46" s="73"/>
-      <c r="I46" s="8"/>
-    </row>
-    <row r="47" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="74"/>
-      <c r="C47" s="75"/>
-      <c r="D47" s="75"/>
-      <c r="E47" s="76"/>
-      <c r="F47" s="63" t="s">
-        <v>50</v>
-      </c>
-      <c r="G47" s="64"/>
-      <c r="H47" s="64"/>
-      <c r="I47" s="65"/>
-    </row>
-    <row r="48" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B48" s="74"/>
-      <c r="C48" s="75"/>
-      <c r="D48" s="75"/>
-      <c r="E48" s="76"/>
-      <c r="F48" s="73" t="s">
-        <v>51</v>
-      </c>
-      <c r="G48" s="73"/>
-      <c r="H48" s="73"/>
-      <c r="I48" s="8"/>
-    </row>
-    <row r="49" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B49" s="77"/>
-      <c r="C49" s="78"/>
-      <c r="D49" s="78"/>
-      <c r="E49" s="79"/>
-      <c r="F49" s="77"/>
-      <c r="G49" s="78"/>
-      <c r="H49" s="78"/>
-      <c r="I49" s="79"/>
-    </row>
-    <row r="50" spans="2:9" ht="9.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B50" s="42"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="18"/>
-      <c r="E50" s="18"/>
-      <c r="F50" s="18"/>
-      <c r="G50" s="18"/>
-      <c r="H50" s="18"/>
-      <c r="I50" s="19"/>
-    </row>
-    <row r="51" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B51" s="56" t="s">
-        <v>22</v>
-      </c>
-      <c r="C51" s="57"/>
-      <c r="D51" s="57"/>
-      <c r="E51" s="57"/>
-      <c r="F51" s="57"/>
-      <c r="G51" s="57"/>
-      <c r="H51" s="57"/>
-      <c r="I51" s="67"/>
-    </row>
-    <row r="52" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B52" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="C52" s="38"/>
-      <c r="D52" s="38"/>
-      <c r="E52" s="38"/>
-      <c r="F52" s="38"/>
-      <c r="G52" s="38"/>
-      <c r="H52" s="38"/>
-      <c r="I52" s="39"/>
-    </row>
-    <row r="53" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B53" s="62"/>
-      <c r="C53" s="62"/>
-      <c r="D53" s="62"/>
-      <c r="E53" s="62"/>
-      <c r="F53" s="62"/>
-      <c r="G53" s="62"/>
-      <c r="H53" s="62"/>
-      <c r="I53" s="62"/>
-    </row>
-    <row r="54" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B54" s="59"/>
-      <c r="C54" s="60"/>
-      <c r="D54" s="60"/>
-      <c r="E54" s="60"/>
-      <c r="F54" s="60"/>
-      <c r="G54" s="60"/>
-      <c r="H54" s="60"/>
-      <c r="I54" s="61"/>
-    </row>
-    <row r="55" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B55" s="56" t="s">
-        <v>24</v>
-      </c>
-      <c r="C55" s="57"/>
-      <c r="D55" s="57"/>
-      <c r="E55" s="57"/>
-      <c r="F55" s="57"/>
-      <c r="G55" s="57"/>
-      <c r="H55" s="57"/>
-      <c r="I55" s="58"/>
-    </row>
-    <row r="56" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B56" s="56"/>
-      <c r="C56" s="57"/>
-      <c r="D56" s="57"/>
-      <c r="E56" s="57"/>
-      <c r="F56" s="57"/>
-      <c r="G56" s="57"/>
-      <c r="H56" s="57"/>
-      <c r="I56" s="58"/>
-    </row>
-    <row r="57" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B57" s="56" t="s">
-        <v>25</v>
-      </c>
-      <c r="C57" s="57"/>
-      <c r="D57" s="57"/>
-      <c r="E57" s="57"/>
-      <c r="F57" s="57"/>
-      <c r="G57" s="57"/>
-      <c r="H57" s="57"/>
-      <c r="I57" s="58"/>
-    </row>
-    <row r="58" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B58" s="56" t="s">
-        <v>26</v>
-      </c>
-      <c r="C58" s="57"/>
-      <c r="D58" s="57"/>
-      <c r="E58" s="57"/>
-      <c r="F58" s="57"/>
-      <c r="G58" s="57"/>
-      <c r="H58" s="57"/>
-      <c r="I58" s="58"/>
-    </row>
-    <row r="59" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B59" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="C59" s="57"/>
-      <c r="D59" s="57"/>
-      <c r="E59" s="57"/>
-      <c r="F59" s="57"/>
-      <c r="G59" s="57"/>
-      <c r="H59" s="57"/>
-      <c r="I59" s="58"/>
-    </row>
-    <row r="60" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B60" s="88"/>
-      <c r="C60" s="89"/>
-      <c r="D60" s="89"/>
-      <c r="E60" s="89"/>
-      <c r="F60" s="89"/>
-      <c r="G60" s="89"/>
-      <c r="H60" s="89"/>
-      <c r="I60" s="90"/>
-    </row>
-    <row r="61" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B61" s="81" t="s">
-        <v>28</v>
-      </c>
-      <c r="C61" s="82"/>
-      <c r="D61" s="83"/>
-      <c r="E61" s="83"/>
-      <c r="F61" s="84" t="s">
-        <v>29</v>
-      </c>
-      <c r="G61" s="84"/>
-      <c r="H61" s="84"/>
-      <c r="I61" s="84"/>
-    </row>
-    <row r="62" spans="2:9" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B62" s="81" t="s">
-        <v>31</v>
-      </c>
-      <c r="C62" s="82"/>
-      <c r="D62" s="83"/>
-      <c r="E62" s="83"/>
-      <c r="F62" s="84" t="s">
-        <v>30</v>
-      </c>
-      <c r="G62" s="84"/>
-      <c r="H62" s="84"/>
-      <c r="I62" s="84"/>
-    </row>
-    <row r="63" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="42"/>
-      <c r="D63" s="83"/>
-      <c r="E63" s="83"/>
-      <c r="F63" s="51" t="s">
-        <v>43</v>
-      </c>
-      <c r="I63" s="50"/>
-    </row>
-    <row r="64" spans="2:9" ht="51.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B64" s="85" t="s">
+      <c r="G68" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="C64" s="86"/>
-      <c r="D64" s="83"/>
-      <c r="E64" s="83"/>
-      <c r="F64" s="87" t="s">
-        <v>40</v>
-      </c>
-      <c r="G64" s="87"/>
-      <c r="H64" s="87"/>
-      <c r="I64" s="87"/>
-    </row>
-    <row r="65" spans="3:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="D65" s="80"/>
-      <c r="E65" s="80"/>
-    </row>
-    <row r="66" spans="3:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="D66" s="80"/>
-      <c r="E66" s="80"/>
-    </row>
-    <row r="68" spans="3:7" x14ac:dyDescent="0.35">
-      <c r="C68" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="G68" s="52" t="s">
-        <v>42</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="65">
+  <mergeCells count="68">
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B6:B9"/>
-    <mergeCell ref="C6:F9"/>
+    <mergeCell ref="C6:G9"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="H7:I7"/>
     <mergeCell ref="H8:I8"/>
@@ -2245,6 +2216,10 @@
     <mergeCell ref="G19:I19"/>
     <mergeCell ref="G21:I21"/>
     <mergeCell ref="B21:F21"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="G30:G31"/>
+    <mergeCell ref="H30:H31"/>
+    <mergeCell ref="I30:I31"/>
     <mergeCell ref="B59:I59"/>
     <mergeCell ref="B60:I60"/>
     <mergeCell ref="B57:I57"/>
@@ -2279,21 +2254,20 @@
     <mergeCell ref="B54:I54"/>
     <mergeCell ref="B53:I53"/>
     <mergeCell ref="F47:I47"/>
-    <mergeCell ref="C33:D33"/>
     <mergeCell ref="B51:I51"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B48:E48"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="B43:I43"/>
     <mergeCell ref="B44:E44"/>
     <mergeCell ref="F44:H44"/>
     <mergeCell ref="B45:E45"/>
     <mergeCell ref="F45:H45"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="B49:E49"/>
-    <mergeCell ref="B48:E48"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="49" orientation="portrait" verticalDpi="300" r:id="rId1"/>
+  <pageSetup scale="48" orientation="portrait" verticalDpi="300" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Arreglos enviados por gabriel 1.0
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO ODC CON BOLIVARES.xlsx
+++ b/storage/app/templates/FORMATO ODC CON BOLIVARES.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\AppData\Roaming\MobaXterm\slash\RemoteFiles\66904_6_4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\AppData\Roaming\MobaXterm\slash\RemoteFiles\132556_2_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09236216-7662-46AB-B395-10165D64E97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2846C0BD-6BC7-41BB-9C20-76EEC800ED33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{CD2C727A-B478-40DC-A0A5-37EBD1630B47}"/>
   </bookViews>
@@ -311,7 +311,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -388,6 +388,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -613,7 +620,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -727,9 +734,213 @@
     <xf numFmtId="4" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -740,210 +951,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1357,54 +1373,54 @@
   </cols>
   <sheetData>
     <row r="6" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="110"/>
-      <c r="C6" s="113" t="s">
+      <c r="B6" s="55"/>
+      <c r="C6" s="124" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="114"/>
-      <c r="E6" s="114"/>
-      <c r="F6" s="114"/>
-      <c r="G6" s="115"/>
-      <c r="H6" s="102" t="s">
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="59"/>
+      <c r="H6" s="66" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="103"/>
+      <c r="I6" s="67"/>
     </row>
     <row r="7" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="111"/>
-      <c r="C7" s="116"/>
-      <c r="D7" s="117"/>
-      <c r="E7" s="117"/>
-      <c r="F7" s="117"/>
-      <c r="G7" s="118"/>
-      <c r="H7" s="102" t="s">
+      <c r="B7" s="56"/>
+      <c r="C7" s="60"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="103"/>
+      <c r="I7" s="67"/>
     </row>
     <row r="8" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="111"/>
-      <c r="C8" s="116"/>
-      <c r="D8" s="117"/>
-      <c r="E8" s="117"/>
-      <c r="F8" s="117"/>
-      <c r="G8" s="118"/>
-      <c r="H8" s="102" t="s">
+      <c r="B8" s="56"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="62"/>
+      <c r="H8" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="I8" s="103"/>
+      <c r="I8" s="67"/>
     </row>
     <row r="9" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="112"/>
-      <c r="C9" s="119"/>
-      <c r="D9" s="120"/>
-      <c r="E9" s="120"/>
-      <c r="F9" s="120"/>
-      <c r="G9" s="121"/>
-      <c r="H9" s="102" t="s">
+      <c r="B9" s="57"/>
+      <c r="C9" s="63"/>
+      <c r="D9" s="64"/>
+      <c r="E9" s="64"/>
+      <c r="F9" s="64"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="66" t="s">
         <v>4</v>
       </c>
-      <c r="I9" s="103"/>
+      <c r="I9" s="67"/>
     </row>
     <row r="10" spans="2:9" ht="21" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
@@ -1417,10 +1433,10 @@
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="2:9" ht="43.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="106" t="s">
+      <c r="B11" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="107"/>
+      <c r="C11" s="50"/>
       <c r="D11" s="15"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
@@ -1429,17 +1445,17 @@
       <c r="I11" s="18"/>
     </row>
     <row r="12" spans="2:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="59" t="s">
+      <c r="B12" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="60"/>
+      <c r="C12" s="52"/>
       <c r="D12" s="19"/>
       <c r="E12" s="20"/>
       <c r="F12" s="21"/>
-      <c r="G12" s="95" t="s">
+      <c r="G12" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="H12" s="95"/>
+      <c r="H12" s="71"/>
       <c r="I12" s="46"/>
     </row>
     <row r="13" spans="2:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.4">
@@ -1450,17 +1466,17 @@
       <c r="D13" s="19"/>
       <c r="E13" s="20"/>
       <c r="F13" s="20"/>
-      <c r="G13" s="95" t="s">
+      <c r="G13" s="71" t="s">
         <v>9</v>
       </c>
-      <c r="H13" s="95"/>
+      <c r="H13" s="71"/>
       <c r="I13" s="46"/>
     </row>
     <row r="14" spans="2:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="59" t="s">
+      <c r="B14" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="60"/>
+      <c r="C14" s="52"/>
       <c r="D14" s="26"/>
       <c r="E14" s="20"/>
       <c r="F14" s="20"/>
@@ -1469,8 +1485,8 @@
       <c r="I14" s="27"/>
     </row>
     <row r="15" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B15" s="108"/>
-      <c r="C15" s="109"/>
+      <c r="B15" s="53"/>
+      <c r="C15" s="54"/>
       <c r="D15" s="28"/>
       <c r="E15" s="22"/>
       <c r="F15" s="22"/>
@@ -1488,10 +1504,10 @@
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
-      <c r="F17" s="104"/>
-      <c r="G17" s="104"/>
-      <c r="H17" s="104"/>
-      <c r="I17" s="105"/>
+      <c r="F17" s="68"/>
+      <c r="G17" s="68"/>
+      <c r="H17" s="68"/>
+      <c r="I17" s="69"/>
     </row>
     <row r="18" spans="2:9" ht="6.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="33"/>
@@ -1511,11 +1527,11 @@
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
       <c r="F19" s="13"/>
-      <c r="G19" s="96" t="s">
+      <c r="G19" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="H19" s="96"/>
-      <c r="I19" s="97"/>
+      <c r="H19" s="72"/>
+      <c r="I19" s="73"/>
     </row>
     <row r="20" spans="2:9" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="33"/>
@@ -1527,18 +1543,18 @@
       <c r="I20" s="10"/>
     </row>
     <row r="21" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="100" t="s">
+      <c r="B21" s="76" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="101"/>
-      <c r="D21" s="101"/>
-      <c r="E21" s="101"/>
-      <c r="F21" s="101"/>
-      <c r="G21" s="98" t="s">
+      <c r="C21" s="77"/>
+      <c r="D21" s="77"/>
+      <c r="E21" s="77"/>
+      <c r="F21" s="77"/>
+      <c r="G21" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="H21" s="98"/>
-      <c r="I21" s="99"/>
+      <c r="H21" s="74"/>
+      <c r="I21" s="75"/>
     </row>
     <row r="22" spans="2:9" ht="12.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="11"/>
@@ -1595,16 +1611,16 @@
       <c r="I26" s="12"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B27" s="92" t="s">
+      <c r="B27" s="90" t="s">
         <v>16</v>
       </c>
-      <c r="C27" s="93"/>
-      <c r="D27" s="93"/>
-      <c r="E27" s="93"/>
-      <c r="F27" s="93"/>
-      <c r="G27" s="93"/>
-      <c r="H27" s="93"/>
-      <c r="I27" s="94"/>
+      <c r="C27" s="91"/>
+      <c r="D27" s="91"/>
+      <c r="E27" s="91"/>
+      <c r="F27" s="91"/>
+      <c r="G27" s="91"/>
+      <c r="H27" s="91"/>
+      <c r="I27" s="92"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B28" s="4"/>
@@ -1627,47 +1643,47 @@
       <c r="I29" s="30"/>
     </row>
     <row r="30" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="87" t="s">
+      <c r="B30" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="C30" s="89" t="s">
+      <c r="C30" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="D30" s="90"/>
-      <c r="E30" s="91" t="s">
+      <c r="D30" s="88"/>
+      <c r="E30" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="F30" s="91" t="s">
+      <c r="F30" s="89" t="s">
         <v>0</v>
       </c>
-      <c r="G30" s="87" t="s">
+      <c r="G30" s="78" t="s">
         <v>50</v>
       </c>
-      <c r="H30" s="87" t="s">
+      <c r="H30" s="78" t="s">
         <v>51</v>
       </c>
-      <c r="I30" s="87" t="s">
+      <c r="I30" s="78" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="31" spans="2:9" ht="45.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="88"/>
-      <c r="C31" s="89"/>
-      <c r="D31" s="90"/>
-      <c r="E31" s="91"/>
-      <c r="F31" s="91"/>
-      <c r="G31" s="88"/>
-      <c r="H31" s="88"/>
-      <c r="I31" s="88"/>
+      <c r="B31" s="79"/>
+      <c r="C31" s="87"/>
+      <c r="D31" s="88"/>
+      <c r="E31" s="89"/>
+      <c r="F31" s="89"/>
+      <c r="G31" s="79"/>
+      <c r="H31" s="79"/>
+      <c r="I31" s="79"/>
     </row>
     <row r="32" spans="2:9" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="49" t="s">
+      <c r="C32" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="D32" s="49"/>
+      <c r="D32" s="70"/>
       <c r="E32" s="37" t="s">
         <v>33</v>
       </c>
@@ -1688,10 +1704,10 @@
       <c r="B33" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="49" t="s">
+      <c r="C33" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="D33" s="49"/>
+      <c r="D33" s="70"/>
       <c r="E33" s="37" t="s">
         <v>33</v>
       </c>
@@ -1712,10 +1728,10 @@
       <c r="B34" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="49" t="s">
+      <c r="C34" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="D34" s="49"/>
+      <c r="D34" s="70"/>
       <c r="E34" s="37" t="s">
         <v>33</v>
       </c>
@@ -1736,10 +1752,10 @@
       <c r="B35" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C35" s="49" t="s">
+      <c r="C35" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="D35" s="49"/>
+      <c r="D35" s="70"/>
       <c r="E35" s="37" t="s">
         <v>33</v>
       </c>
@@ -1760,10 +1776,10 @@
       <c r="B36" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C36" s="49" t="s">
+      <c r="C36" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="D36" s="49"/>
+      <c r="D36" s="70"/>
       <c r="E36" s="37" t="s">
         <v>33</v>
       </c>
@@ -1784,10 +1800,10 @@
       <c r="B37" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C37" s="49" t="s">
+      <c r="C37" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="D37" s="49"/>
+      <c r="D37" s="70"/>
       <c r="E37" s="37" t="s">
         <v>33</v>
       </c>
@@ -1808,10 +1824,10 @@
       <c r="B38" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C38" s="49" t="s">
+      <c r="C38" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="D38" s="49"/>
+      <c r="D38" s="70"/>
       <c r="E38" s="37" t="s">
         <v>33</v>
       </c>
@@ -1832,10 +1848,10 @@
       <c r="B39" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="49" t="s">
+      <c r="C39" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="D39" s="49"/>
+      <c r="D39" s="70"/>
       <c r="E39" s="37" t="s">
         <v>33</v>
       </c>
@@ -1856,10 +1872,10 @@
       <c r="B40" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C40" s="49" t="s">
+      <c r="C40" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="D40" s="49"/>
+      <c r="D40" s="70"/>
       <c r="E40" s="37" t="s">
         <v>33</v>
       </c>
@@ -1880,10 +1896,10 @@
       <c r="B41" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C41" s="49" t="s">
+      <c r="C41" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="D41" s="49"/>
+      <c r="D41" s="70"/>
       <c r="E41" s="37" t="s">
         <v>33</v>
       </c>
@@ -1904,10 +1920,10 @@
       <c r="B42" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C42" s="49" t="s">
+      <c r="C42" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="D42" s="49"/>
+      <c r="D42" s="70"/>
       <c r="E42" s="37" t="s">
         <v>33</v>
       </c>
@@ -1925,86 +1941,86 @@
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B43" s="50"/>
-      <c r="C43" s="50"/>
-      <c r="D43" s="50"/>
-      <c r="E43" s="50"/>
-      <c r="F43" s="50"/>
-      <c r="G43" s="50"/>
-      <c r="H43" s="50"/>
-      <c r="I43" s="50"/>
+      <c r="B43" s="118"/>
+      <c r="C43" s="118"/>
+      <c r="D43" s="118"/>
+      <c r="E43" s="118"/>
+      <c r="F43" s="118"/>
+      <c r="G43" s="118"/>
+      <c r="H43" s="118"/>
+      <c r="I43" s="118"/>
     </row>
     <row r="44" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B44" s="51"/>
-      <c r="C44" s="52"/>
-      <c r="D44" s="52"/>
-      <c r="E44" s="52"/>
-      <c r="F44" s="53" t="s">
+      <c r="B44" s="119"/>
+      <c r="C44" s="120"/>
+      <c r="D44" s="120"/>
+      <c r="E44" s="120"/>
+      <c r="F44" s="104" t="s">
         <v>43</v>
       </c>
-      <c r="G44" s="54"/>
-      <c r="H44" s="55"/>
+      <c r="G44" s="105"/>
+      <c r="H44" s="106"/>
       <c r="I44" s="7"/>
     </row>
     <row r="45" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B45" s="53" t="s">
+      <c r="B45" s="121" t="s">
         <v>48</v>
       </c>
-      <c r="C45" s="55"/>
-      <c r="D45" s="55"/>
-      <c r="E45" s="55"/>
-      <c r="F45" s="53" t="s">
+      <c r="C45" s="122"/>
+      <c r="D45" s="122"/>
+      <c r="E45" s="123"/>
+      <c r="F45" s="104" t="s">
         <v>44</v>
       </c>
-      <c r="G45" s="54"/>
-      <c r="H45" s="55"/>
+      <c r="G45" s="105"/>
+      <c r="H45" s="106"/>
       <c r="I45" s="7"/>
     </row>
     <row r="46" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B46" s="70"/>
-      <c r="C46" s="71"/>
-      <c r="D46" s="71"/>
-      <c r="E46" s="72"/>
-      <c r="F46" s="53" t="s">
+      <c r="B46" s="121"/>
+      <c r="C46" s="122"/>
+      <c r="D46" s="122"/>
+      <c r="E46" s="123"/>
+      <c r="F46" s="104" t="s">
         <v>45</v>
       </c>
-      <c r="G46" s="54"/>
-      <c r="H46" s="55"/>
+      <c r="G46" s="105"/>
+      <c r="H46" s="106"/>
       <c r="I46" s="7"/>
     </row>
     <row r="47" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="70"/>
-      <c r="C47" s="71"/>
-      <c r="D47" s="71"/>
-      <c r="E47" s="72"/>
-      <c r="F47" s="66" t="s">
+      <c r="B47" s="115"/>
+      <c r="C47" s="116"/>
+      <c r="D47" s="116"/>
+      <c r="E47" s="117"/>
+      <c r="F47" s="111" t="s">
         <v>46</v>
       </c>
-      <c r="G47" s="67"/>
-      <c r="H47" s="67"/>
-      <c r="I47" s="68"/>
+      <c r="G47" s="112"/>
+      <c r="H47" s="112"/>
+      <c r="I47" s="113"/>
     </row>
     <row r="48" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B48" s="70"/>
-      <c r="C48" s="71"/>
-      <c r="D48" s="71"/>
-      <c r="E48" s="72"/>
-      <c r="F48" s="55" t="s">
+      <c r="B48" s="115"/>
+      <c r="C48" s="116"/>
+      <c r="D48" s="116"/>
+      <c r="E48" s="117"/>
+      <c r="F48" s="106" t="s">
         <v>47</v>
       </c>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
+      <c r="G48" s="106"/>
+      <c r="H48" s="106"/>
       <c r="I48" s="7"/>
     </row>
     <row r="49" spans="2:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B49" s="56"/>
-      <c r="C49" s="57"/>
-      <c r="D49" s="57"/>
-      <c r="E49" s="58"/>
-      <c r="F49" s="56"/>
-      <c r="G49" s="57"/>
-      <c r="H49" s="57"/>
-      <c r="I49" s="58"/>
+      <c r="B49" s="101"/>
+      <c r="C49" s="102"/>
+      <c r="D49" s="102"/>
+      <c r="E49" s="103"/>
+      <c r="F49" s="101"/>
+      <c r="G49" s="102"/>
+      <c r="H49" s="102"/>
+      <c r="I49" s="103"/>
     </row>
     <row r="50" spans="2:9" ht="9.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B50" s="39"/>
@@ -2017,16 +2033,16 @@
       <c r="I50" s="18"/>
     </row>
     <row r="51" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B51" s="59" t="s">
+      <c r="B51" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="C51" s="60"/>
-      <c r="D51" s="60"/>
-      <c r="E51" s="60"/>
-      <c r="F51" s="60"/>
-      <c r="G51" s="60"/>
-      <c r="H51" s="60"/>
-      <c r="I51" s="69"/>
+      <c r="C51" s="52"/>
+      <c r="D51" s="52"/>
+      <c r="E51" s="52"/>
+      <c r="F51" s="52"/>
+      <c r="G51" s="52"/>
+      <c r="H51" s="52"/>
+      <c r="I51" s="114"/>
     </row>
     <row r="52" spans="2:9" ht="21" x14ac:dyDescent="0.4">
       <c r="B52" s="34" t="s">
@@ -2041,82 +2057,82 @@
       <c r="I52" s="36"/>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B53" s="65"/>
-      <c r="C53" s="65"/>
-      <c r="D53" s="65"/>
-      <c r="E53" s="65"/>
-      <c r="F53" s="65"/>
-      <c r="G53" s="65"/>
-      <c r="H53" s="65"/>
-      <c r="I53" s="65"/>
+      <c r="B53" s="110"/>
+      <c r="C53" s="110"/>
+      <c r="D53" s="110"/>
+      <c r="E53" s="110"/>
+      <c r="F53" s="110"/>
+      <c r="G53" s="110"/>
+      <c r="H53" s="110"/>
+      <c r="I53" s="110"/>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B54" s="62"/>
-      <c r="C54" s="63"/>
-      <c r="D54" s="63"/>
-      <c r="E54" s="63"/>
-      <c r="F54" s="63"/>
-      <c r="G54" s="63"/>
-      <c r="H54" s="63"/>
-      <c r="I54" s="64"/>
+      <c r="B54" s="107"/>
+      <c r="C54" s="108"/>
+      <c r="D54" s="108"/>
+      <c r="E54" s="108"/>
+      <c r="F54" s="108"/>
+      <c r="G54" s="108"/>
+      <c r="H54" s="108"/>
+      <c r="I54" s="109"/>
     </row>
     <row r="55" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B55" s="59" t="s">
+      <c r="B55" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C55" s="60"/>
-      <c r="D55" s="60"/>
-      <c r="E55" s="60"/>
-      <c r="F55" s="60"/>
-      <c r="G55" s="60"/>
-      <c r="H55" s="60"/>
-      <c r="I55" s="61"/>
+      <c r="C55" s="52"/>
+      <c r="D55" s="52"/>
+      <c r="E55" s="52"/>
+      <c r="F55" s="52"/>
+      <c r="G55" s="52"/>
+      <c r="H55" s="52"/>
+      <c r="I55" s="80"/>
     </row>
     <row r="56" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B56" s="59"/>
-      <c r="C56" s="60"/>
-      <c r="D56" s="60"/>
-      <c r="E56" s="60"/>
-      <c r="F56" s="60"/>
-      <c r="G56" s="60"/>
-      <c r="H56" s="60"/>
-      <c r="I56" s="61"/>
+      <c r="B56" s="51"/>
+      <c r="C56" s="52"/>
+      <c r="D56" s="52"/>
+      <c r="E56" s="52"/>
+      <c r="F56" s="52"/>
+      <c r="G56" s="52"/>
+      <c r="H56" s="52"/>
+      <c r="I56" s="80"/>
     </row>
     <row r="57" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B57" s="59" t="s">
+      <c r="B57" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="C57" s="60"/>
-      <c r="D57" s="60"/>
-      <c r="E57" s="60"/>
-      <c r="F57" s="60"/>
-      <c r="G57" s="60"/>
-      <c r="H57" s="60"/>
-      <c r="I57" s="61"/>
+      <c r="C57" s="52"/>
+      <c r="D57" s="52"/>
+      <c r="E57" s="52"/>
+      <c r="F57" s="52"/>
+      <c r="G57" s="52"/>
+      <c r="H57" s="52"/>
+      <c r="I57" s="80"/>
     </row>
     <row r="58" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B58" s="59" t="s">
+      <c r="B58" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="C58" s="60"/>
-      <c r="D58" s="60"/>
-      <c r="E58" s="60"/>
-      <c r="F58" s="60"/>
-      <c r="G58" s="60"/>
-      <c r="H58" s="60"/>
-      <c r="I58" s="61"/>
+      <c r="C58" s="52"/>
+      <c r="D58" s="52"/>
+      <c r="E58" s="52"/>
+      <c r="F58" s="52"/>
+      <c r="G58" s="52"/>
+      <c r="H58" s="52"/>
+      <c r="I58" s="80"/>
     </row>
     <row r="59" spans="2:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="B59" s="59" t="s">
+      <c r="B59" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="C59" s="60"/>
-      <c r="D59" s="60"/>
-      <c r="E59" s="60"/>
-      <c r="F59" s="60"/>
-      <c r="G59" s="60"/>
-      <c r="H59" s="60"/>
-      <c r="I59" s="61"/>
+      <c r="C59" s="52"/>
+      <c r="D59" s="52"/>
+      <c r="E59" s="52"/>
+      <c r="F59" s="52"/>
+      <c r="G59" s="52"/>
+      <c r="H59" s="52"/>
+      <c r="I59" s="80"/>
     </row>
     <row r="60" spans="2:9" ht="21" x14ac:dyDescent="0.35">
       <c r="B60" s="81"/>
@@ -2129,63 +2145,63 @@
       <c r="I60" s="83"/>
     </row>
     <row r="61" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B61" s="74" t="s">
+      <c r="B61" s="94" t="s">
         <v>26</v>
       </c>
-      <c r="C61" s="75"/>
-      <c r="D61" s="76"/>
-      <c r="E61" s="76"/>
-      <c r="F61" s="77" t="s">
+      <c r="C61" s="95"/>
+      <c r="D61" s="96"/>
+      <c r="E61" s="96"/>
+      <c r="F61" s="97" t="s">
         <v>27</v>
       </c>
-      <c r="G61" s="77"/>
-      <c r="H61" s="77"/>
-      <c r="I61" s="77"/>
+      <c r="G61" s="97"/>
+      <c r="H61" s="97"/>
+      <c r="I61" s="97"/>
     </row>
     <row r="62" spans="2:9" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B62" s="74" t="s">
+      <c r="B62" s="94" t="s">
         <v>29</v>
       </c>
-      <c r="C62" s="75"/>
-      <c r="D62" s="76"/>
-      <c r="E62" s="76"/>
-      <c r="F62" s="77" t="s">
+      <c r="C62" s="95"/>
+      <c r="D62" s="96"/>
+      <c r="E62" s="96"/>
+      <c r="F62" s="97" t="s">
         <v>28</v>
       </c>
-      <c r="G62" s="77"/>
-      <c r="H62" s="77"/>
-      <c r="I62" s="77"/>
+      <c r="G62" s="97"/>
+      <c r="H62" s="97"/>
+      <c r="I62" s="97"/>
     </row>
     <row r="63" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B63" s="39"/>
-      <c r="D63" s="76"/>
-      <c r="E63" s="76"/>
+      <c r="D63" s="96"/>
+      <c r="E63" s="96"/>
       <c r="F63" s="44" t="s">
         <v>41</v>
       </c>
       <c r="I63" s="43"/>
     </row>
     <row r="64" spans="2:9" ht="51.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B64" s="78" t="s">
+      <c r="B64" s="98" t="s">
         <v>38</v>
       </c>
-      <c r="C64" s="79"/>
-      <c r="D64" s="76"/>
-      <c r="E64" s="76"/>
-      <c r="F64" s="80" t="s">
+      <c r="C64" s="99"/>
+      <c r="D64" s="96"/>
+      <c r="E64" s="96"/>
+      <c r="F64" s="100" t="s">
         <v>38</v>
       </c>
-      <c r="G64" s="80"/>
-      <c r="H64" s="80"/>
-      <c r="I64" s="80"/>
+      <c r="G64" s="100"/>
+      <c r="H64" s="100"/>
+      <c r="I64" s="100"/>
     </row>
     <row r="65" spans="3:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="D65" s="73"/>
-      <c r="E65" s="73"/>
+      <c r="D65" s="93"/>
+      <c r="E65" s="93"/>
     </row>
     <row r="66" spans="3:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="D66" s="73"/>
-      <c r="E66" s="73"/>
+      <c r="D66" s="93"/>
+      <c r="E66" s="93"/>
     </row>
     <row r="68" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C68" s="17" t="s">
@@ -2196,30 +2212,35 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="68">
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="C6:G9"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="G30:G31"/>
-    <mergeCell ref="H30:H31"/>
-    <mergeCell ref="I30:I31"/>
+  <mergeCells count="67">
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="F44:H44"/>
+    <mergeCell ref="F45:H45"/>
+    <mergeCell ref="B45:E46"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="F46:H46"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="B56:I56"/>
+    <mergeCell ref="B58:I58"/>
+    <mergeCell ref="B55:I55"/>
+    <mergeCell ref="B54:I54"/>
+    <mergeCell ref="B53:I53"/>
+    <mergeCell ref="F47:I47"/>
+    <mergeCell ref="B51:I51"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="D61:E64"/>
+    <mergeCell ref="F61:I61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="F62:I62"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="F64:I64"/>
     <mergeCell ref="B59:I59"/>
     <mergeCell ref="B60:I60"/>
     <mergeCell ref="B57:I57"/>
@@ -2236,35 +2257,29 @@
     <mergeCell ref="C37:D37"/>
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="C35:D35"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="D61:E64"/>
-    <mergeCell ref="F61:I61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="F62:I62"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="F64:I64"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="F46:H46"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="B56:I56"/>
-    <mergeCell ref="B58:I58"/>
-    <mergeCell ref="B55:I55"/>
-    <mergeCell ref="B54:I54"/>
-    <mergeCell ref="B53:I53"/>
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="B51:I51"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="B49:E49"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="B43:I43"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="F44:H44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="F45:H45"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="G30:G31"/>
+    <mergeCell ref="H30:H31"/>
+    <mergeCell ref="I30:I31"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="C6:G9"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="48" orientation="portrait" verticalDpi="300" r:id="rId1"/>

</xml_diff>